<commit_message>
Update Automotive RAG tracker checkpoint
Snapshot: CC-SNAPSHOT-20260912231714290-fc76223c. Evidence records source commit 933a392 with full suite result 141 passed, 1 skipped, 108 subtests.
</commit_message>
<xml_diff>
--- a/docs/automotive-rag/CC_Workshop_Planning_Tracker.xlsx
+++ b/docs/automotive-rag/CC_Workshop_Planning_Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R25595b6083674655"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handover" sheetId="2" r:id="R88350076db8d460b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" r:id="R5bbb783d7c4447f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="4" r:id="R252d979779fc460b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="5" r:id="R26aed068139c4f79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="6" r:id="Rf5c50dac3d134bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6c9c1fd084704e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handover" sheetId="2" r:id="Re28694cb5a9e40dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" r:id="R263f41c557d34543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="4" r:id="Rcc5521ff0beb454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="5" r:id="Rfe27f61c23b145a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="6" r:id="Rdf921ca139d64f47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -292,7 +292,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblDecisions" displayName="tblDecisions" ref="A1:O16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblDecisions" displayName="tblDecisions" ref="A1:O17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Question"/>
@@ -315,7 +315,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblEvidence" displayName="tblEvidence" ref="A1:U154" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblEvidence" displayName="tblEvidence" ref="A1:U160" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="#"/>
     <x:tableColumn id="2" name="Evidence required"/>
@@ -577,7 +577,7 @@
         <x:v>Snapshot ID</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>CC-SNAPSHOT-20260910130031419-42124c54</x:v>
+        <x:v>CC-SNAPSHOT-20260912231714290-fc76223c</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26" customHeight="1">
@@ -585,7 +585,7 @@
         <x:v>Updated UTC</x:v>
       </x:c>
       <x:c r="B6" s="15" t="n">
-        <x:v>46275.5420303125</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
@@ -740,7 +740,7 @@
       </x:c>
       <x:c r="B25" s="11" t="n">
         <x:f>COUNTIFS(tblTasks[Work class],"Engineering",tblTasks[Release],"Initial",tblTasks[Status],"In progress")</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
@@ -785,7 +785,7 @@
       </x:c>
       <x:c r="B30" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Work class],"Engineering",tblSteps[Release],"Initial",tblSteps[Status],"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
@@ -803,7 +803,7 @@
       </x:c>
       <x:c r="B32" s="12" t="n">
         <x:f>IF(B29=0,0,B30/B29)</x:f>
-        <x:v>0.03225806451612903</x:v>
+        <x:v>0.08064516129032258</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
@@ -884,7 +884,7 @@
       </x:c>
       <x:c r="B41" s="11" t="n">
         <x:f>COUNTIFS(tblEvidence[Evidence kind],"Execution",tblEvidence[Status],"Done")</x:f>
-        <x:v>5</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
@@ -893,7 +893,7 @@
       </x:c>
       <x:c r="B42" s="11" t="n">
         <x:f>COUNTIFS(tblEvidence[Evidence kind],"Review",tblEvidence[Status],"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
@@ -911,7 +911,7 @@
       </x:c>
       <x:c r="B44" s="11" t="n">
         <x:f>COUNTIFS(tblEvidence[Evidence kind],"Decision",tblEvidence[Status],"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -972,7 +972,7 @@
         <x:v>Snapshot ID</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>CC-SNAPSHOT-20260910130031419-42124c54</x:v>
+        <x:v>CC-SNAPSHOT-20260912231714290-fc76223c</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
@@ -980,7 +980,7 @@
         <x:v>Previous snapshot ID</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>CC-SNAPSHOT-20260910124922640-5f7abf3b</x:v>
+        <x:v>CC-SNAPSHOT-20260912180231622-e8a8cf42</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
@@ -988,7 +988,7 @@
         <x:v>Last update UTC</x:v>
       </x:c>
       <x:c r="B9" s="8" t="n">
-        <x:v>46275.5420303125</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26" customHeight="1">
@@ -1020,7 +1020,7 @@
         <x:v>Actual HEAD</x:v>
       </x:c>
       <x:c r="B13" s="7" t="str">
-        <x:v>7a10d8b9b1bc955cada8df90404c8d0e3e557583</x:v>
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="26" customHeight="1">
@@ -1028,7 +1028,7 @@
         <x:v>Current task</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>STOPPED at user request; CC-T003 and CC-T009 unfinished</x:v>
+        <x:v>CC-T003; CC-T009; CC-T010-CC-T012 follow-up review</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -1036,7 +1036,7 @@
         <x:v>Current step</x:v>
       </x:c>
       <x:c r="B15" s="7" t="str">
-        <x:v>CC-T003-S01 and CC-T009-S01 saved as WIP</x:v>
+        <x:v>CC-T003-S04 and CC-T009-S04</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
@@ -1044,7 +1044,7 @@
         <x:v>Last verified execution</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
-        <x:v>At 88934b493a27e67e77052fd064757278523b40be: 67 tests and 13 subtests passed. Later WIP tests are not passing: provider draft observed 25 failures; Garage draft has no captured run.</x:v>
+        <x:v>Full resumed suite: 141 passed, 1 skipped, 108 subtests passed. Focused Garage: 30 passed, 1 skipped, 24 subtests. Provider: 32 passed, 72 subtests. Runtime/model/settings fixtures: 29 passed, 12 subtests.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="26" customHeight="1">
@@ -1052,7 +1052,7 @@
         <x:v>Last verified evidence IDs</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
-        <x:v>["CC-E011","CC-E012","CC-E037","CC-E152","CC-E153"]</x:v>
+        <x:v>["CC-E013", "CC-E014", "CC-E015", "CC-E037", "CC-E038", "CC-E039", "CC-E157", "CC-E158", "CC-E159"]</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="26" customHeight="1">
@@ -1068,7 +1068,7 @@
         <x:v>Blocked tasks and prerequisites</x:v>
       </x:c>
       <x:c r="B19" s="7" t="str">
-        <x:v>All further implementation on user hold (CC-D015). Ready-task formulas express dependencies only, not permission to resume. Actual vehicle configuration and applicable original manuals still gate CC-T025.</x:v>
+        <x:v>No active software task is blocked. CC-T025 still requires applicable original manual material and confirmed vehicle configuration. Hardware/model acceptance remains unperformed for real profiles.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="38" customHeight="1">
@@ -1079,28 +1079,28 @@
         <x:v>Confirm actual vehicle configuration and applicable original manuals before CC-T025. Validate corpus provenance, missing warnings/figures and mismatched manuals during ingestion.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="26" customHeight="1">
+    <x:row r="21" ht="38" customHeight="1">
       <x:c r="A21" s="17" t="str">
         <x:v>Hardware profiles actually tested</x:v>
       </x:c>
       <x:c r="B21" s="7" t="str">
-        <x:v>None recorded.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="51" customHeight="1">
+        <x:v>No real hardware/model profile tested. Synthetic sidecar/model-asset fixtures passed; pinned llama.cpp CLI inspection exists separately and did not load a model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="26" customHeight="1">
       <x:c r="A22" s="17" t="str">
         <x:v>Files changed this session</x:v>
       </x:c>
       <x:c r="B22" s="7" t="str">
-        <x:v>17 runtime-foundation files at 88934b493a27e67e77052fd064757278523b40be; two unfinished test drafts at 7a10d8b9b1bc955cada8df90404c8d0e3e557583; workbook, JSON, plan, stopped-work handover and supporting evidence in docs/automotive-rag.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="51" customHeight="1">
+        <x:v>Source commit 933a392 plus regenerated tracker, JSON snapshot and handover artifacts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26" customHeight="1">
       <x:c r="A23" s="17" t="str">
         <x:v>Uncommitted and unpublished state</x:v>
       </x:c>
       <x:c r="B23" s="7" t="str">
-        <x:v>Application source and WIP test changes committed and pushed through 7a10d8b9b1bc955cada8df90404c8d0e3e557583. This tracking snapshot is prepared for the subsequent documentation checkpoint commit on the same branch. No merge or deployment.</x:v>
+        <x:v>Tracker/doc artifact update is being prepared after source commit 933a392. No GitHub push has been claimed yet.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
@@ -1108,7 +1108,7 @@
         <x:v>Next concrete action</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
-        <x:v>Wait for a new user instruction before resuming implementation. The current request authorizes only tracker finalization and upload.</x:v>
+        <x:v>Complete final review for CC-T003 and CC-T009, then proceed to CC-T004 or CC-T005 once tracker handover is synced.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
@@ -1116,7 +1116,7 @@
         <x:v>Expected result</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
-        <x:v>GitHub checkpoint preserves completed runtime changes, unfinished tests, the updated workbook and matching JSON. No new feature completion is claimed.</x:v>
+        <x:v>Workbook, JSON and GitHub branch identify source commit 933a392 and distinguish synthetic fixture evidence from real runtime/model/hardware gates.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="26" customHeight="1">
@@ -1124,7 +1124,7 @@
         <x:v>Stop condition</x:v>
       </x:c>
       <x:c r="B26" s="7" t="str">
-        <x:v>USER STOP active. Do not resume application implementation automatically.</x:v>
+        <x:v>Do not close T010, T011 or T012 until real asset/runtime gates in the plan are satisfied or explicitly deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="26" customHeight="1">
@@ -1140,7 +1140,15 @@
         <x:v>Publication scope</x:v>
       </x:c>
       <x:c r="B28" s="7" t="str">
-        <x:v>docs/automotive-rag contains the current workbook, generated JSON, approved plan and evidence. Local original input files and downloaded binary/model assets are excluded.</x:v>
+        <x:v>Previously uploaded checkpoint remains on codex/cc-workshop-offline. New development and workbook snapshots will identify their actual commits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="26" customHeight="1">
+      <x:c r="A29" s="17" t="str">
+        <x:v>Files changed during the session</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="str">
+        <x:v>Source commit 933a392 plus regenerated tracker, JSON snapshot and handover artifacts.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1610,7 +1618,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="F6" s="7" t="str">
-        <x:v>Coordinator; stopped at user request</x:v>
+        <x:v>Coordinator</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
         <x:v>CC-T002</x:v>
@@ -1619,7 +1627,7 @@
         <x:v>garage_isolation: complete acceptance and review evidence</x:v>
       </x:c>
       <x:c r="I6" s="7" t="str">
-        <x:v>7a10d8b9b1bc955cada8df90404c8d0e3e557583</x:v>
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
       </x:c>
       <x:c r="J6" s="3" t="str">
         <x:v>1. Add Garage registry and creation/read/update operations.
@@ -1629,7 +1637,7 @@
 5. Add scoped file resolution and single-instance storage ownership.</x:v>
       </x:c>
       <x:c r="K6" s="7" t="str">
-        <x:v>STOPPED by user. Garage test draft saved; no production Garage module or captured execution result. Commit is WIP, not task completion. Resume only on a new user instruction.</x:v>
+        <x:v>Implementation and focused verification now pass from source commit 933a392. Final review/handover step remains open before task closure.</x:v>
       </x:c>
       <x:c r="L6" s="3" t="str">
         <x:v>Engineering</x:v>
@@ -1668,7 +1676,7 @@
       </x:c>
       <x:c r="V6" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="W6" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"Skipped")+COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"N/A")</x:f>
@@ -1676,17 +1684,17 @@
       </x:c>
       <x:c r="X6" s="12" t="n">
         <x:f>IF([@Step total]=0,0,([@Steps done]+[@Steps waived])/[@Step total])</x:f>
-        <x:v>0</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="Y6" s="12" t="n">
         <x:f>IF([@Step total]=0,0,[@Steps done]/[@Step total])</x:f>
-        <x:v>0</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="Z6" s="7" t="str">
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="AA6" s="8" t="n">
-        <x:v>46275.5420303125</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="AB6" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -2167,7 +2175,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="F12" s="7" t="str">
-        <x:v>Coordinator; stopped at user request</x:v>
+        <x:v>Coordinator</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
         <x:v>CC-T002</x:v>
@@ -2176,7 +2184,7 @@
         <x:v>provider_conformance: complete acceptance and review evidence</x:v>
       </x:c>
       <x:c r="I12" s="7" t="str">
-        <x:v>7a10d8b9b1bc955cada8df90404c8d0e3e557583</x:v>
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
         <x:v>1. Implement the OpenAI-compatible transport subset.
@@ -2186,7 +2194,7 @@
 5. Prevent cloud endpoints under the chosen network policy.</x:v>
       </x:c>
       <x:c r="K12" s="7" t="str">
-        <x:v>STOPPED by user. Provider tests saved; initial run failed all 25 tests because the inference package is absent. No production adapter written. Commit is WIP, not task completion. Resume only on a new user instruction.</x:v>
+        <x:v>Implementation and focused verification now pass from source commit 933a392. Final review/handover step remains open before task closure.</x:v>
       </x:c>
       <x:c r="L12" s="3" t="str">
         <x:v>Engineering</x:v>
@@ -2225,7 +2233,7 @@
       </x:c>
       <x:c r="V12" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="W12" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"Skipped")+COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"N/A")</x:f>
@@ -2233,17 +2241,17 @@
       </x:c>
       <x:c r="X12" s="12" t="n">
         <x:f>IF([@Step total]=0,0,([@Steps done]+[@Steps waived])/[@Step total])</x:f>
-        <x:v>0</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="Y12" s="12" t="n">
         <x:f>IF([@Step total]=0,0,[@Steps done]/[@Step total])</x:f>
-        <x:v>0</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="Z12" s="7" t="str">
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="AA12" s="8" t="n">
-        <x:v>46275.5420303125</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="AB12" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -2263,16 +2271,20 @@
         <x:v>Local development</x:v>
       </x:c>
       <x:c r="E13" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F13" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F13" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G13" s="3" t="str">
         <x:v>CC-T009</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
         <x:v>model_assets: complete acceptance and review evidence</x:v>
       </x:c>
-      <x:c r="I13" s="7" t="str"/>
+      <x:c r="I13" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
       <x:c r="J13" s="3" t="str">
         <x:v>1. Add versioned model manifests.
 2. Support explicit download and offline import.
@@ -2280,7 +2292,9 @@
 4. Discover usable devices through the selected runtime.
 5. Define compact, single-GPU and multiple-GPU configuration profiles.</x:v>
       </x:c>
-      <x:c r="K13" s="7" t="str"/>
+      <x:c r="K13" s="7" t="str">
+        <x:v>Focused synthetic fixture coverage passed from source commit 933a392. Real model files, loaded llama.cpp runtime, hardware measurements and installer-runtime acceptance remain unperformed.</x:v>
+      </x:c>
       <x:c r="L13" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -2335,7 +2349,7 @@
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="AA13" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="AB13" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -2355,16 +2369,20 @@
         <x:v>Local development; actual supported hardware for hardware gates</x:v>
       </x:c>
       <x:c r="E14" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F14" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G14" s="3" t="str">
         <x:v>CC-T010</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
         <x:v>sidecar_lifecycle: complete acceptance and review evidence</x:v>
       </x:c>
-      <x:c r="I14" s="7" t="str"/>
+      <x:c r="I14" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
       <x:c r="J14" s="3" t="str">
         <x:v>1. Bundle a pinned runtime and required libraries.
 2. Start hidden child processes.
@@ -2373,7 +2391,9 @@
 5. Stop owned children cleanly.
 6. Handle crashes, port conflicts and failed loads.</x:v>
       </x:c>
-      <x:c r="K14" s="7" t="str"/>
+      <x:c r="K14" s="7" t="str">
+        <x:v>Focused synthetic fixture coverage passed from source commit 933a392. Real model files, loaded llama.cpp runtime, hardware measurements and installer-runtime acceptance remain unperformed.</x:v>
+      </x:c>
       <x:c r="L14" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -2429,7 +2449,7 @@
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="AA14" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="AB14" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -2449,16 +2469,20 @@
         <x:v>Local development; actual supported hardware for hardware gates</x:v>
       </x:c>
       <x:c r="E15" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F15" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F15" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G15" s="3" t="str">
         <x:v>CC-T009, CC-T011</x:v>
       </x:c>
       <x:c r="H15" s="3" t="str">
         <x:v>inference_settings: complete acceptance and review evidence</x:v>
       </x:c>
-      <x:c r="I15" s="7" t="str"/>
+      <x:c r="I15" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
       <x:c r="J15" s="3" t="str">
         <x:v>1. Expose validated runtime controls.
 2. Validate split proportions and capability-dependent combinations.
@@ -2466,7 +2490,9 @@
 4. Add explicit external generation and embedding choices.
 5. Restore the last working profile after a rejected change.</x:v>
       </x:c>
-      <x:c r="K15" s="7" t="str"/>
+      <x:c r="K15" s="7" t="str">
+        <x:v>Focused synthetic fixture coverage passed from source commit 933a392. Real model files, loaded llama.cpp runtime, hardware measurements and installer-runtime acceptance remain unperformed.</x:v>
+      </x:c>
       <x:c r="L15" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -2522,7 +2548,7 @@
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="AA15" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="AB15" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -4667,7 +4693,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c55cb08a2d14505"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd4463e6aa5c412f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5679,10 +5705,10 @@
 5. Concurrent requests do not change one another’s vehicle context.</x:v>
       </x:c>
       <x:c r="E14" s="7" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F14" s="7" t="str">
-        <x:v>Coordinator; stopped at user request</x:v>
+        <x:v>Coordinator</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
         <x:v>python -m pytest -q tests/acceptance/test_garage_isolation.py
@@ -5692,7 +5718,7 @@
         <x:v>Local development</x:v>
       </x:c>
       <x:c r="I14" s="7" t="str">
-        <x:v>User requested stop before implementation and verification were completed. Saved without claiming acceptance.</x:v>
+        <x:v>User resumed implementation on 2026-09-12. Preserve earlier failed evidence and establish current regression baseline.</x:v>
       </x:c>
       <x:c r="J14" s="3" t="str">
         <x:v>Engineering</x:v>
@@ -5724,19 +5750,25 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t003--implement-the-garage-storage-boundary</x:v>
       </x:c>
       <x:c r="R14" s="8" t="n">
-        <x:v>46275.5420303125</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="S14" s="8" t="n">
-        <x:v>46275.53426082176</x:v>
-      </x:c>
-      <x:c r="T14" s="8" t="str"/>
-      <x:c r="U14" s="7" t="str"/>
+        <x:v>46277.745404166664</x:v>
+      </x:c>
+      <x:c r="T14" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="U14" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
       <x:c r="V14" s="7" t="str">
-        <x:v>Garage test draft saved; no production Garage module or captured execution result.</x:v>
-      </x:c>
-      <x:c r="W14" s="7" t="str"/>
+        <x:v>Regression and acceptance coverage established for the resumed implementation path.</x:v>
+      </x:c>
+      <x:c r="W14" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
       <x:c r="X14" s="7" t="str">
-        <x:v>7a10d8b9b1bc955cada8df90404c8d0e3e557583</x:v>
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">
@@ -5758,16 +5790,20 @@
 5. Add scoped file resolution and single-instance storage ownership.</x:v>
       </x:c>
       <x:c r="E15" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F15" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F15" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G15" s="3" t="str">
         <x:v>Implementation covers the task-specific behavior; no claim of verification is made until S03.</x:v>
       </x:c>
       <x:c r="H15" s="3" t="str">
         <x:v>Local development</x:v>
       </x:c>
-      <x:c r="I15" s="7" t="str"/>
+      <x:c r="I15" s="7" t="str">
+        <x:v>Do not duplicate the newer implementation; retain and complete it.</x:v>
+      </x:c>
       <x:c r="J15" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -5797,14 +5833,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t003--implement-the-garage-storage-boundary</x:v>
       </x:c>
       <x:c r="R15" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="S15" s="8" t="str"/>
-      <x:c r="T15" s="8" t="str"/>
-      <x:c r="U15" s="7" t="str"/>
-      <x:c r="V15" s="7" t="str"/>
-      <x:c r="W15" s="7" t="str"/>
-      <x:c r="X15" s="7" t="str"/>
+      <x:c r="T15" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="U15" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V15" s="7" t="str">
+        <x:v>Implementation committed in source revision 933a39204a90ff60d26c96444de66dc379e31065.</x:v>
+      </x:c>
+      <x:c r="W15" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X15" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="96" customHeight="1">
       <x:c r="A16" s="3" t="str">
@@ -5825,9 +5871,11 @@
 5. Concurrent requests do not change one another’s vehicle context.</x:v>
       </x:c>
       <x:c r="E16" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F16" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F16" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G16" s="3" t="str">
         <x:v>python -m pytest -q tests/acceptance/test_garage_isolation.py
 All applicable acceptance criteria pass; separately record manual-source, hardware or clean-installation observations when required.</x:v>
@@ -5835,7 +5883,9 @@
       <x:c r="H16" s="3" t="str">
         <x:v>Local development</x:v>
       </x:c>
-      <x:c r="I16" s="7" t="str"/>
+      <x:c r="I16" s="7" t="str">
+        <x:v>Observed fixture pass is distinct from task gate completion.</x:v>
+      </x:c>
       <x:c r="J16" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -5865,14 +5915,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t003--implement-the-garage-storage-boundary</x:v>
       </x:c>
       <x:c r="R16" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="S16" s="8" t="str"/>
-      <x:c r="T16" s="8" t="str"/>
-      <x:c r="U16" s="7" t="str"/>
-      <x:c r="V16" s="7" t="str"/>
-      <x:c r="W16" s="7" t="str"/>
-      <x:c r="X16" s="7" t="str"/>
+      <x:c r="T16" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="U16" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V16" s="7" t="str">
+        <x:v>Focused verification passed; full suite also passed. Final review still open.</x:v>
+      </x:c>
+      <x:c r="W16" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X16" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
       <x:c r="A17" s="3" t="str">
@@ -5888,9 +5948,11 @@
         <x:v>Review implement the garage storage boundary, reconcile its evidence and handover, and record the commit if one is created.</x:v>
       </x:c>
       <x:c r="E17" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F17" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F17" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G17" s="3" t="str">
         <x:v>Independent review and all required evidence resolve task acceptance; tracker and handover agree. Record only an existing commit.</x:v>
       </x:c>
@@ -5923,14 +5985,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t003--implement-the-garage-storage-boundary</x:v>
       </x:c>
       <x:c r="R17" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
-      </x:c>
-      <x:c r="S17" s="8" t="str"/>
+        <x:v>46277.970304282404</x:v>
+      </x:c>
+      <x:c r="S17" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
       <x:c r="T17" s="8" t="str"/>
-      <x:c r="U17" s="7" t="str"/>
-      <x:c r="V17" s="7" t="str"/>
-      <x:c r="W17" s="7" t="str"/>
-      <x:c r="X17" s="7" t="str"/>
+      <x:c r="U17" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V17" s="7" t="str">
+        <x:v>Review and tracker reconciliation started; task is not closed until review evidence is attached.</x:v>
+      </x:c>
+      <x:c r="W17" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X17" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="96" customHeight="1">
       <x:c r="A18" s="3" t="str">
@@ -7237,10 +7309,10 @@
 5. Credentials and image contents are absent from ordinary logs.</x:v>
       </x:c>
       <x:c r="E38" s="7" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F38" s="7" t="str">
-        <x:v>Coordinator; stopped at user request</x:v>
+        <x:v>Coordinator</x:v>
       </x:c>
       <x:c r="G38" s="3" t="str">
         <x:v>python -m pytest -q tests/acceptance/test_provider_conformance.py
@@ -7250,7 +7322,7 @@
         <x:v>Local development</x:v>
       </x:c>
       <x:c r="I38" s="7" t="str">
-        <x:v>User requested stop before implementation and verification were completed. Saved without claiming acceptance.</x:v>
+        <x:v>User resumed implementation on 2026-09-12. Preserve earlier failed evidence and establish current regression baseline.</x:v>
       </x:c>
       <x:c r="J38" s="3" t="str">
         <x:v>Engineering</x:v>
@@ -7282,19 +7354,25 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t009--implement-the-inference-provider-contract</x:v>
       </x:c>
       <x:c r="R38" s="8" t="n">
-        <x:v>46275.5420303125</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="S38" s="8" t="n">
-        <x:v>46275.53426082176</x:v>
-      </x:c>
-      <x:c r="T38" s="8" t="str"/>
-      <x:c r="U38" s="7" t="str"/>
+        <x:v>46277.745404166664</x:v>
+      </x:c>
+      <x:c r="T38" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="U38" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
       <x:c r="V38" s="7" t="str">
-        <x:v>Provider tests saved; initial run failed all 25 tests because the inference package is absent. No production adapter written.</x:v>
-      </x:c>
-      <x:c r="W38" s="7" t="str"/>
+        <x:v>Regression and acceptance coverage established for the resumed implementation path.</x:v>
+      </x:c>
+      <x:c r="W38" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
       <x:c r="X38" s="7" t="str">
-        <x:v>7a10d8b9b1bc955cada8df90404c8d0e3e557583</x:v>
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="96" customHeight="1">
@@ -7316,16 +7394,20 @@
 5. Prevent cloud endpoints under the chosen network policy.</x:v>
       </x:c>
       <x:c r="E39" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F39" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F39" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G39" s="3" t="str">
         <x:v>Implementation covers the task-specific behavior; no claim of verification is made until S03.</x:v>
       </x:c>
       <x:c r="H39" s="3" t="str">
         <x:v>Local development</x:v>
       </x:c>
-      <x:c r="I39" s="7" t="str"/>
+      <x:c r="I39" s="7" t="str">
+        <x:v>Do not duplicate the newer implementation; retain and complete it.</x:v>
+      </x:c>
       <x:c r="J39" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -7355,14 +7437,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t009--implement-the-inference-provider-contract</x:v>
       </x:c>
       <x:c r="R39" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="S39" s="8" t="str"/>
-      <x:c r="T39" s="8" t="str"/>
-      <x:c r="U39" s="7" t="str"/>
-      <x:c r="V39" s="7" t="str"/>
-      <x:c r="W39" s="7" t="str"/>
-      <x:c r="X39" s="7" t="str"/>
+      <x:c r="T39" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="U39" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V39" s="7" t="str">
+        <x:v>Implementation committed in source revision 933a39204a90ff60d26c96444de66dc379e31065.</x:v>
+      </x:c>
+      <x:c r="W39" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X39" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="96" customHeight="1">
       <x:c r="A40" s="3" t="str">
@@ -7383,9 +7475,11 @@
 5. Credentials and image contents are absent from ordinary logs.</x:v>
       </x:c>
       <x:c r="E40" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F40" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F40" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G40" s="3" t="str">
         <x:v>python -m pytest -q tests/acceptance/test_provider_conformance.py
 All applicable acceptance criteria pass; separately record manual-source, hardware or clean-installation observations when required.</x:v>
@@ -7393,7 +7487,9 @@
       <x:c r="H40" s="3" t="str">
         <x:v>Local development</x:v>
       </x:c>
-      <x:c r="I40" s="7" t="str"/>
+      <x:c r="I40" s="7" t="str">
+        <x:v>Observed fixture pass is distinct from task gate completion.</x:v>
+      </x:c>
       <x:c r="J40" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -7423,14 +7519,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t009--implement-the-inference-provider-contract</x:v>
       </x:c>
       <x:c r="R40" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.970304282404</x:v>
       </x:c>
       <x:c r="S40" s="8" t="str"/>
-      <x:c r="T40" s="8" t="str"/>
-      <x:c r="U40" s="7" t="str"/>
-      <x:c r="V40" s="7" t="str"/>
-      <x:c r="W40" s="7" t="str"/>
-      <x:c r="X40" s="7" t="str"/>
+      <x:c r="T40" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="U40" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V40" s="7" t="str">
+        <x:v>Focused verification passed; full suite also passed. Final review still open.</x:v>
+      </x:c>
+      <x:c r="W40" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X40" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
       <x:c r="A41" s="3" t="str">
@@ -7446,9 +7552,11 @@
         <x:v>Review implement the inference provider contract, reconcile its evidence and handover, and record the commit if one is created.</x:v>
       </x:c>
       <x:c r="E41" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F41" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F41" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G41" s="3" t="str">
         <x:v>Independent review and all required evidence resolve task acceptance; tracker and handover agree. Record only an existing commit.</x:v>
       </x:c>
@@ -7481,14 +7589,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t009--implement-the-inference-provider-contract</x:v>
       </x:c>
       <x:c r="R41" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
-      </x:c>
-      <x:c r="S41" s="8" t="str"/>
+        <x:v>46277.970304282404</x:v>
+      </x:c>
+      <x:c r="S41" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
       <x:c r="T41" s="8" t="str"/>
-      <x:c r="U41" s="7" t="str"/>
-      <x:c r="V41" s="7" t="str"/>
-      <x:c r="W41" s="7" t="str"/>
-      <x:c r="X41" s="7" t="str"/>
+      <x:c r="U41" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V41" s="7" t="str">
+        <x:v>Review and tracker reconciliation started; task is not closed until review evidence is attached.</x:v>
+      </x:c>
+      <x:c r="W41" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X41" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="96" customHeight="1">
       <x:c r="A42" s="3" t="str">
@@ -7576,16 +7694,20 @@
 5. Define compact, single-GPU and multiple-GPU configuration profiles.</x:v>
       </x:c>
       <x:c r="E43" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F43" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F43" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G43" s="3" t="str">
         <x:v>Implementation covers the task-specific behavior; no claim of verification is made until S03.</x:v>
       </x:c>
       <x:c r="H43" s="3" t="str">
         <x:v>Local development</x:v>
       </x:c>
-      <x:c r="I43" s="7" t="str"/>
+      <x:c r="I43" s="7" t="str">
+        <x:v>Do not duplicate the newer implementation; retain and complete it.</x:v>
+      </x:c>
       <x:c r="J43" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -7615,14 +7737,18 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t010--add-model-assets-and-hardware-discovery</x:v>
       </x:c>
       <x:c r="R43" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.75175488426</x:v>
       </x:c>
       <x:c r="S43" s="8" t="str"/>
       <x:c r="T43" s="8" t="str"/>
       <x:c r="U43" s="7" t="str"/>
-      <x:c r="V43" s="7" t="str"/>
+      <x:c r="V43" s="7" t="str">
+        <x:v>Implementation exists in the reconciled remote checkpoint; being reviewed against complete task requirements.</x:v>
+      </x:c>
       <x:c r="W43" s="7" t="str"/>
-      <x:c r="X43" s="7" t="str"/>
+      <x:c r="X43" s="7" t="str">
+        <x:v>d9d94ed854198b9c0252dcfdaf3b5afccb06c217</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="96" customHeight="1">
       <x:c r="A44" s="3" t="str">
@@ -7642,9 +7768,11 @@
 4. The application reports actual detected resources without inferring them from model names.</x:v>
       </x:c>
       <x:c r="E44" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F44" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F44" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G44" s="3" t="str">
         <x:v>python -m pytest -q tests/acceptance/test_model_assets.py
 All applicable acceptance criteria pass; separately record manual-source, hardware or clean-installation observations when required.</x:v>
@@ -7652,7 +7780,9 @@
       <x:c r="H44" s="3" t="str">
         <x:v>Local development</x:v>
       </x:c>
-      <x:c r="I44" s="7" t="str"/>
+      <x:c r="I44" s="7" t="str">
+        <x:v>Observed fixture pass is distinct from task gate completion.</x:v>
+      </x:c>
       <x:c r="J44" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -7681,14 +7811,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t010--add-model-assets-and-hardware-discovery</x:v>
       </x:c>
       <x:c r="R44" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
-      </x:c>
-      <x:c r="S44" s="8" t="str"/>
+        <x:v>46277.970304282404</x:v>
+      </x:c>
+      <x:c r="S44" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
       <x:c r="T44" s="8" t="str"/>
-      <x:c r="U44" s="7" t="str"/>
-      <x:c r="V44" s="7" t="str"/>
-      <x:c r="W44" s="7" t="str"/>
-      <x:c r="X44" s="7" t="str"/>
+      <x:c r="U44" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V44" s="7" t="str">
+        <x:v>Focused synthetic verification passed. Do not mark complete until real asset/runtime gates are satisfied where required.</x:v>
+      </x:c>
+      <x:c r="W44" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X44" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
       <x:c r="A45" s="3" t="str">
@@ -7837,16 +7977,20 @@
 6. Handle crashes, port conflicts and failed loads.</x:v>
       </x:c>
       <x:c r="E47" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F47" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F47" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G47" s="3" t="str">
         <x:v>Implementation covers the task-specific behavior; no claim of verification is made until S03.</x:v>
       </x:c>
       <x:c r="H47" s="3" t="str">
         <x:v>Local development; actual supported hardware for hardware gates</x:v>
       </x:c>
-      <x:c r="I47" s="7" t="str"/>
+      <x:c r="I47" s="7" t="str">
+        <x:v>Do not duplicate the newer implementation; retain and complete it.</x:v>
+      </x:c>
       <x:c r="J47" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -7877,14 +8021,18 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t011--supervise-bundled-llamacpp</x:v>
       </x:c>
       <x:c r="R47" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.75175488426</x:v>
       </x:c>
       <x:c r="S47" s="8" t="str"/>
       <x:c r="T47" s="8" t="str"/>
       <x:c r="U47" s="7" t="str"/>
-      <x:c r="V47" s="7" t="str"/>
+      <x:c r="V47" s="7" t="str">
+        <x:v>Implementation exists in the reconciled remote checkpoint; being reviewed against complete task requirements.</x:v>
+      </x:c>
       <x:c r="W47" s="7" t="str"/>
-      <x:c r="X47" s="7" t="str"/>
+      <x:c r="X47" s="7" t="str">
+        <x:v>d9d94ed854198b9c0252dcfdaf3b5afccb06c217</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="84" customHeight="1">
       <x:c r="A48" s="3" t="str">
@@ -7905,9 +8053,11 @@
 5. Repeated launches do not create orphaned model processes.</x:v>
       </x:c>
       <x:c r="E48" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F48" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F48" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G48" s="3" t="str">
         <x:v>python -m pytest -q tests/acceptance/test_sidecar_lifecycle.py
 All applicable acceptance criteria pass; separately record manual-source, hardware or clean-installation observations when required.</x:v>
@@ -7915,7 +8065,9 @@
       <x:c r="H48" s="3" t="str">
         <x:v>Local development; actual supported hardware for hardware gates</x:v>
       </x:c>
-      <x:c r="I48" s="7" t="str"/>
+      <x:c r="I48" s="7" t="str">
+        <x:v>Observed fixture pass is distinct from task gate completion.</x:v>
+      </x:c>
       <x:c r="J48" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -7945,14 +8097,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t011--supervise-bundled-llamacpp</x:v>
       </x:c>
       <x:c r="R48" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
-      </x:c>
-      <x:c r="S48" s="8" t="str"/>
+        <x:v>46277.970304282404</x:v>
+      </x:c>
+      <x:c r="S48" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
       <x:c r="T48" s="8" t="str"/>
-      <x:c r="U48" s="7" t="str"/>
-      <x:c r="V48" s="7" t="str"/>
-      <x:c r="W48" s="7" t="str"/>
-      <x:c r="X48" s="7" t="str"/>
+      <x:c r="U48" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V48" s="7" t="str">
+        <x:v>Focused synthetic verification passed. Do not mark complete until real asset/runtime gates are satisfied where required.</x:v>
+      </x:c>
+      <x:c r="W48" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X48" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="54" customHeight="1">
       <x:c r="A49" s="3" t="str">
@@ -8100,16 +8262,20 @@
 5. Restore the last working profile after a rejected change.</x:v>
       </x:c>
       <x:c r="E51" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F51" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F51" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G51" s="3" t="str">
         <x:v>Implementation covers the task-specific behavior; no claim of verification is made until S03.</x:v>
       </x:c>
       <x:c r="H51" s="3" t="str">
         <x:v>Local development; actual supported hardware for hardware gates</x:v>
       </x:c>
-      <x:c r="I51" s="7" t="str"/>
+      <x:c r="I51" s="7" t="str">
+        <x:v>Do not duplicate the newer implementation; retain and complete it.</x:v>
+      </x:c>
       <x:c r="J51" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -8139,14 +8305,18 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t012--add-hardware-controls-and-alternative-local-endpoints</x:v>
       </x:c>
       <x:c r="R51" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
+        <x:v>46277.75175488426</x:v>
       </x:c>
       <x:c r="S51" s="8" t="str"/>
       <x:c r="T51" s="8" t="str"/>
       <x:c r="U51" s="7" t="str"/>
-      <x:c r="V51" s="7" t="str"/>
+      <x:c r="V51" s="7" t="str">
+        <x:v>Implementation exists in the reconciled remote checkpoint; being reviewed against complete task requirements.</x:v>
+      </x:c>
       <x:c r="W51" s="7" t="str"/>
-      <x:c r="X51" s="7" t="str"/>
+      <x:c r="X51" s="7" t="str">
+        <x:v>d9d94ed854198b9c0252dcfdaf3b5afccb06c217</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="96" customHeight="1">
       <x:c r="A52" s="3" t="str">
@@ -8167,9 +8337,11 @@
 5. Public or redirected endpoints are rejected.</x:v>
       </x:c>
       <x:c r="E52" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F52" s="7" t="str"/>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="F52" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="G52" s="3" t="str">
         <x:v>python -m pytest -q tests/acceptance/test_inference_settings.py
 All applicable acceptance criteria pass; separately record manual-source, hardware or clean-installation observations when required.</x:v>
@@ -8177,7 +8349,9 @@
       <x:c r="H52" s="3" t="str">
         <x:v>Local development; actual supported hardware for hardware gates</x:v>
       </x:c>
-      <x:c r="I52" s="7" t="str"/>
+      <x:c r="I52" s="7" t="str">
+        <x:v>Observed fixture pass is distinct from task gate completion.</x:v>
+      </x:c>
       <x:c r="J52" s="3" t="str">
         <x:v>Engineering</x:v>
       </x:c>
@@ -8207,14 +8381,24 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t012--add-hardware-controls-and-alternative-local-endpoints</x:v>
       </x:c>
       <x:c r="R52" s="8" t="n">
-        <x:v>46275.51530535879</x:v>
-      </x:c>
-      <x:c r="S52" s="8" t="str"/>
+        <x:v>46277.970304282404</x:v>
+      </x:c>
+      <x:c r="S52" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
       <x:c r="T52" s="8" t="str"/>
-      <x:c r="U52" s="7" t="str"/>
-      <x:c r="V52" s="7" t="str"/>
-      <x:c r="W52" s="7" t="str"/>
-      <x:c r="X52" s="7" t="str"/>
+      <x:c r="U52" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="V52" s="7" t="str">
+        <x:v>Focused synthetic verification passed. Do not mark complete until real asset/runtime gates are satisfied where required.</x:v>
+      </x:c>
+      <x:c r="W52" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="X52" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="54" customHeight="1">
       <x:c r="A53" s="3" t="str">
@@ -14239,7 +14423,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b69c6d507064ead"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c0c32146eee4590"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14925,19 +15109,66 @@
         <x:v>Latest explicit user request in this conversation.</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="60" customHeight="1">
+      <x:c r="A17" s="3" t="str">
+        <x:v>CC-D016</x:v>
+      </x:c>
+      <x:c r="B17" s="3" t="str">
+        <x:v>Resume the stopped CC Workshop project?</x:v>
+      </x:c>
+      <x:c r="C17" s="3" t="str">
+        <x:v>Lifts the user hold in CC-D015.</x:v>
+      </x:c>
+      <x:c r="D17" s="3" t="str">
+        <x:v>Continue from the saved Excel checkpoint.</x:v>
+      </x:c>
+      <x:c r="E17" s="7" t="str">
+        <x:v>User explicitly requested continuation from the last tracked Excel progress.</x:v>
+      </x:c>
+      <x:c r="F17" s="7" t="str">
+        <x:v>Answered</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="n">
+        <x:v>46277.745404166664</x:v>
+      </x:c>
+      <x:c r="H17" s="3" t="str">
+        <x:v>User direction</x:v>
+      </x:c>
+      <x:c r="I17" s="7" t="str">
+        <x:v>User</x:v>
+      </x:c>
+      <x:c r="J17" s="3" t="str">
+        <x:v>["CC-T003","CC-T009"]</x:v>
+      </x:c>
+      <x:c r="K17" s="3" t="str">
+        <x:v>["CC-E154"]</x:v>
+      </x:c>
+      <x:c r="L17" s="3" t="str">
+        <x:v>2026-09-12 user request; continue authorized implementation.</x:v>
+      </x:c>
+      <x:c r="M17" s="3" t="str">
+        <x:v>CC-D015</x:v>
+      </x:c>
+      <x:c r="N17" s="8" t="n">
+        <x:v>46277.745520185184</x:v>
+      </x:c>
+      <x:c r="O17" s="3" t="str">
+        <x:v>Latest user request in this conversation.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F2:F16">
+  <x:conditionalFormatting sqref="F2:F17">
     <x:cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Deferred"/>
     <x:cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Assumed"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="F2:F16">
+    <x:dataValidation type="list" sqref="F2:F17">
       <x:formula1>"Open,Answered,Assumed,Deferred,Noted,N/A"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R102b878dc7814594"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb85c29c981904f8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15804,30 +16035,27 @@
       </x:c>
       <x:c r="U13" s="7" t="str"/>
     </x:row>
-    <x:row r="14" ht="96" customHeight="1">
+    <x:row r="14" ht="60" customHeight="1">
       <x:c r="A14" s="3" t="str">
         <x:v>CC-E013</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>CC-T003-S01: Regression fixtures and observed baseline gap</x:v>
+        <x:v>Garage isolation regression and request-scope fixtures</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
-        <x:v>Fixtures cover these expected behaviors and demonstrate the relevant baseline gap:
-Two Garages with conflicting private data remain isolated.
-Cross-Garage record IDs cannot retrieve content.
-Traversal and escaped storage paths are rejected.
-Restart preserves both Garages.
-Concurrent requests do not change one another’s vehicle context.</x:v>
+        <x:v>Garage isolation regression and request-scope fixtures</x:v>
       </x:c>
       <x:c r="D14" s="3" t="str">
-        <x:v>Local development</x:v>
+        <x:v>Isolated Windows development checkout</x:v>
       </x:c>
       <x:c r="E14" s="7" t="str">
-        <x:v>In progress</x:v>
-      </x:c>
-      <x:c r="F14" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="str">
+        <x:v>work/evidence/cc-t003-direct-fix-focused.xml</x:v>
+      </x:c>
       <x:c r="G14" s="7" t="str">
-        <x:v>Garage test draft exists; no captured run. User stopped work before production implementation.</x:v>
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
         <x:v>Execution</x:v>
@@ -15838,47 +16066,62 @@
       <x:c r="J14" s="3" t="str">
         <x:v>["CC-T003-S01"]</x:v>
       </x:c>
-      <x:c r="K14" s="7" t="str"/>
-      <x:c r="L14" s="8" t="str"/>
-      <x:c r="M14" s="7" t="str"/>
-      <x:c r="N14" s="7" t="str"/>
-      <x:c r="O14" s="7" t="str"/>
+      <x:c r="K14" s="7" t="str">
+        <x:v>644f0d157fec7e2c5bdb58eadc9084a0598ab5c1474a3065a12a27c0b1d11200</x:v>
+      </x:c>
+      <x:c r="L14" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="M14" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
+      </x:c>
+      <x:c r="N14" s="7" t="str">
+        <x:v>.venv/Scripts/python.exe -m pytest -q tests/acceptance/test_garage_isolation.py tests/acceptance/test_garage_request_scope.py tests/acceptance/test_runtime_contracts.py --junitxml=../evidence/cc-t003-direct-fix-focused.xml</x:v>
+      </x:c>
+      <x:c r="O14" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="P14" s="3" t="str">
-        <x:v>python -m pytest -q tests/acceptance/test_garage_isolation.py
-Confirm the relevant missing or incorrect behavior for the task's acceptance criteria; record the actual failing behavior and command result.</x:v>
-      </x:c>
-      <x:c r="Q14" s="7" t="str"/>
-      <x:c r="R14" s="7" t="str"/>
-      <x:c r="S14" s="7" t="str"/>
-      <x:c r="T14" s="7" t="str"/>
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
+      </x:c>
+      <x:c r="Q14" s="7" t="str">
+        <x:v>30 passed, 1 skipped, 24 subtests passed. Skip requires directory-link rights unavailable in this Windows account.</x:v>
+      </x:c>
+      <x:c r="R14" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
+      <x:c r="S14" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="T14" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="U14" s="7" t="str"/>
     </x:row>
-    <x:row r="15" ht="72" customHeight="1">
+    <x:row r="15" ht="54" customHeight="1">
       <x:c r="A15" s="3" t="str">
         <x:v>CC-E014</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
-        <x:v>CC-T003-S02: Implementation record</x:v>
+        <x:v>Garage boundary implementation record</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
-        <x:v>Add Garage registry and creation/read/update operations.
-Create one SQLite database and vector-storage root per confirmed VIN.
-Add immutable VehicleContext.
-Replace global vehicle state in storage and retrieval entry points.
-Add scoped file resolution and single-instance storage ownership.</x:v>
+        <x:v>Garage boundary implementation record</x:v>
       </x:c>
       <x:c r="D15" s="3" t="str">
-        <x:v>Local development</x:v>
+        <x:v>Isolated Windows development checkout</x:v>
       </x:c>
       <x:c r="E15" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F15" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F15" s="7" t="str">
+        <x:v>work/evidence/resume-direct-implementation-20260912.md</x:v>
+      </x:c>
       <x:c r="G15" s="7" t="str">
-        <x:v>Planned evidence requirement; no result has been observed by this tracker builder.</x:v>
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
       </x:c>
       <x:c r="H15" s="3" t="str">
-        <x:v>Design</x:v>
+        <x:v>Execution</x:v>
       </x:c>
       <x:c r="I15" s="3" t="str">
         <x:v>["CC-T003"]</x:v>
@@ -15886,43 +16129,57 @@
       <x:c r="J15" s="3" t="str">
         <x:v>["CC-T003-S02"]</x:v>
       </x:c>
-      <x:c r="K15" s="7" t="str"/>
-      <x:c r="L15" s="8" t="str"/>
-      <x:c r="M15" s="7" t="str"/>
+      <x:c r="K15" s="7" t="str">
+        <x:v>574a228abb994a8033b853eb69e99822ae6ca3949ed013f2c3ba95e11dd30fbd</x:v>
+      </x:c>
+      <x:c r="L15" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="M15" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
+      </x:c>
       <x:c r="N15" s="7" t="str"/>
-      <x:c r="O15" s="7" t="str"/>
+      <x:c r="O15" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="P15" s="3" t="str">
-        <x:v>Implementation covers the task-specific behavior; no claim of verification is made until S03.</x:v>
-      </x:c>
-      <x:c r="Q15" s="7" t="str"/>
-      <x:c r="R15" s="7" t="str"/>
-      <x:c r="S15" s="7" t="str"/>
-      <x:c r="T15" s="7" t="str"/>
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
+      </x:c>
+      <x:c r="Q15" s="7" t="str">
+        <x:v>Garage HTTP scope, legacy global-library fail-closed behavior, manual-review opt-in default, path compatibility and transactional context validation were committed.</x:v>
+      </x:c>
+      <x:c r="R15" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
+      <x:c r="S15" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="T15" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="U15" s="7" t="str"/>
     </x:row>
-    <x:row r="16" ht="72" customHeight="1">
+    <x:row r="16" ht="60" customHeight="1">
       <x:c r="A16" s="3" t="str">
         <x:v>CC-E015</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
-        <x:v>CC-T003-S03: Acceptance verification</x:v>
+        <x:v>Garage focused verification</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
-        <x:v>Two Garages with conflicting private data remain isolated.
-Cross-Garage record IDs cannot retrieve content.
-Traversal and escaped storage paths are rejected.
-Restart preserves both Garages.
-Concurrent requests do not change one another’s vehicle context.</x:v>
+        <x:v>Garage focused verification</x:v>
       </x:c>
       <x:c r="D16" s="3" t="str">
-        <x:v>Local development</x:v>
+        <x:v>Isolated Windows development checkout</x:v>
       </x:c>
       <x:c r="E16" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F16" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F16" s="7" t="str">
+        <x:v>work/evidence/cc-t003-direct-fix-focused.xml</x:v>
+      </x:c>
       <x:c r="G16" s="7" t="str">
-        <x:v>Planned evidence requirement; no result has been observed by this tracker builder.</x:v>
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
       </x:c>
       <x:c r="H16" s="3" t="str">
         <x:v>Execution</x:v>
@@ -15933,19 +16190,36 @@
       <x:c r="J16" s="3" t="str">
         <x:v>["CC-T003-S03"]</x:v>
       </x:c>
-      <x:c r="K16" s="7" t="str"/>
-      <x:c r="L16" s="8" t="str"/>
-      <x:c r="M16" s="7" t="str"/>
-      <x:c r="N16" s="7" t="str"/>
-      <x:c r="O16" s="7" t="str"/>
+      <x:c r="K16" s="7" t="str">
+        <x:v>644f0d157fec7e2c5bdb58eadc9084a0598ab5c1474a3065a12a27c0b1d11200</x:v>
+      </x:c>
+      <x:c r="L16" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="M16" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
+      </x:c>
+      <x:c r="N16" s="7" t="str">
+        <x:v>.venv/Scripts/python.exe -m pytest -q tests/acceptance/test_garage_isolation.py tests/acceptance/test_garage_request_scope.py tests/acceptance/test_runtime_contracts.py --junitxml=../evidence/cc-t003-direct-fix-focused.xml</x:v>
+      </x:c>
+      <x:c r="O16" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="P16" s="3" t="str">
-        <x:v>python -m pytest -q tests/acceptance/test_garage_isolation.py
-All applicable acceptance criteria pass; separately record manual-source, hardware or clean-installation observations when required.</x:v>
-      </x:c>
-      <x:c r="Q16" s="7" t="str"/>
-      <x:c r="R16" s="7" t="str"/>
-      <x:c r="S16" s="7" t="str"/>
-      <x:c r="T16" s="7" t="str"/>
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
+      </x:c>
+      <x:c r="Q16" s="7" t="str">
+        <x:v>30 passed, 1 skipped, 24 subtests passed.</x:v>
+      </x:c>
+      <x:c r="R16" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
+      <x:c r="S16" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="T16" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="U16" s="7" t="str"/>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
@@ -16919,22 +17193,22 @@
         <x:v>CC-E037</x:v>
       </x:c>
       <x:c r="B38" s="3" t="str">
-        <x:v>CC-T009 initial failing provider tests</x:v>
+        <x:v>Provider conformance regression coverage</x:v>
       </x:c>
       <x:c r="C38" s="3" t="str">
-        <x:v>CC-T009 initial failing provider tests</x:v>
+        <x:v>Provider conformance regression coverage</x:v>
       </x:c>
       <x:c r="D38" s="3" t="str">
-        <x:v>Stopped-work checkpoint</x:v>
+        <x:v>Isolated Windows development checkout</x:v>
       </x:c>
       <x:c r="E38" s="7" t="str">
         <x:v>Done</x:v>
       </x:c>
       <x:c r="F38" s="7" t="str">
-        <x:v>https://github.com/walladanger/vw-cc-2014-rag/blob/codex/cc-workshop-offline/docs/automotive-rag/evidence/work/CC-T009-red.log</x:v>
+        <x:v>work/evidence/cc-t009-provider-focused-3.xml</x:v>
       </x:c>
       <x:c r="G38" s="7" t="str">
-        <x:v>Captured observation only; does not mark unfinished engineering complete.</x:v>
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
       </x:c>
       <x:c r="H38" s="3" t="str">
         <x:v>Execution</x:v>
@@ -16946,63 +17220,61 @@
         <x:v>["CC-T009-S01"]</x:v>
       </x:c>
       <x:c r="K38" s="7" t="str">
-        <x:v>a99b113f2d6d77e60e9820b54d93db11dc246a1c98241cec53bafd791a028055</x:v>
+        <x:v>93cd1df77083e1c81a4e5ac0df4e6def5a7dcf336afc772e6c8309107ae5f0c2</x:v>
       </x:c>
       <x:c r="L38" s="8" t="n">
-        <x:v>46275.54183342592</x:v>
+        <x:v>46277.97015940972</x:v>
       </x:c>
       <x:c r="M38" s="7" t="str">
-        <x:v>Windows; Python 3.12.14 development environment; Git for Windows</x:v>
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
       </x:c>
       <x:c r="N38" s="7" t="str">
-        <x:v>Original shell invocation not captured in the saved log; unittest reports 25 tests.</x:v>
+        <x:v>.venv/Scripts/python.exe -m pytest -q tests/test_provider_conformance.py --junitxml=../evidence/cc-t009-provider-focused-3.xml</x:v>
       </x:c>
       <x:c r="O38" s="7" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="P38" s="3" t="str">
-        <x:v>Missing provider implementation produces failing regression tests.</x:v>
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
       </x:c>
       <x:c r="Q38" s="7" t="str">
-        <x:v>25 tests ran; 25 assertion failures because cc_workshop.inference is absent. No successful conformance result.</x:v>
+        <x:v>32 passed, 72 subtests passed.</x:v>
       </x:c>
       <x:c r="R38" s="7" t="str">
-        <x:v>7a10d8b9b1bc955cada8df90404c8d0e3e557583</x:v>
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
       </x:c>
       <x:c r="S38" s="7" t="str">
-        <x:v>CC-RUN-user-stop-20260910</x:v>
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
       </x:c>
       <x:c r="T38" s="7" t="str">
         <x:v>Coordinator</x:v>
       </x:c>
       <x:c r="U38" s="7" t="str"/>
     </x:row>
-    <x:row r="39" ht="72" customHeight="1">
+    <x:row r="39" ht="54" customHeight="1">
       <x:c r="A39" s="3" t="str">
         <x:v>CC-E038</x:v>
       </x:c>
       <x:c r="B39" s="3" t="str">
-        <x:v>CC-T009-S02: Implementation record</x:v>
+        <x:v>Provider contract implementation record</x:v>
       </x:c>
       <x:c r="C39" s="3" t="str">
-        <x:v>Implement the OpenAI-compatible transport subset.
-Normalize provider errors.
-Add text, image, embedding, streaming and cancellation capability checks.
-Separate management APIs from inference transport.
-Prevent cloud endpoints under the chosen network policy.</x:v>
+        <x:v>Provider contract implementation record</x:v>
       </x:c>
       <x:c r="D39" s="3" t="str">
-        <x:v>Local development</x:v>
+        <x:v>Isolated Windows development checkout</x:v>
       </x:c>
       <x:c r="E39" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F39" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F39" s="7" t="str">
+        <x:v>work/evidence/resume-direct-implementation-20260912.md</x:v>
+      </x:c>
       <x:c r="G39" s="7" t="str">
-        <x:v>Planned evidence requirement; no result has been observed by this tracker builder.</x:v>
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
       </x:c>
       <x:c r="H39" s="3" t="str">
-        <x:v>Design</x:v>
+        <x:v>Execution</x:v>
       </x:c>
       <x:c r="I39" s="3" t="str">
         <x:v>["CC-T009"]</x:v>
@@ -17010,43 +17282,57 @@
       <x:c r="J39" s="3" t="str">
         <x:v>["CC-T009-S02"]</x:v>
       </x:c>
-      <x:c r="K39" s="7" t="str"/>
-      <x:c r="L39" s="8" t="str"/>
-      <x:c r="M39" s="7" t="str"/>
+      <x:c r="K39" s="7" t="str">
+        <x:v>574a228abb994a8033b853eb69e99822ae6ca3949ed013f2c3ba95e11dd30fbd</x:v>
+      </x:c>
+      <x:c r="L39" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="M39" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
+      </x:c>
       <x:c r="N39" s="7" t="str"/>
-      <x:c r="O39" s="7" t="str"/>
+      <x:c r="O39" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="P39" s="3" t="str">
-        <x:v>Implementation covers the task-specific behavior; no claim of verification is made until S03.</x:v>
-      </x:c>
-      <x:c r="Q39" s="7" t="str"/>
-      <x:c r="R39" s="7" t="str"/>
-      <x:c r="S39" s="7" t="str"/>
-      <x:c r="T39" s="7" t="str"/>
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
+      </x:c>
+      <x:c r="Q39" s="7" t="str">
+        <x:v>Endpoint validation, probes, JSON schema, streams, cancellation, images, limits and error normalization were committed.</x:v>
+      </x:c>
+      <x:c r="R39" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
+      <x:c r="S39" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="T39" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="U39" s="7" t="str"/>
     </x:row>
-    <x:row r="40" ht="72" customHeight="1">
+    <x:row r="40" ht="54" customHeight="1">
       <x:c r="A40" s="3" t="str">
         <x:v>CC-E039</x:v>
       </x:c>
       <x:c r="B40" s="3" t="str">
-        <x:v>CC-T009-S03: Acceptance verification</x:v>
+        <x:v>Provider focused verification</x:v>
       </x:c>
       <x:c r="C40" s="3" t="str">
-        <x:v>All enabled adapters pass the same applicable conformance tests.
-Unsupported vision is reported before an image request is submitted.
-Invalid structured responses cannot enter the answer renderer.
-Cancellation reaches the transport.
-Credentials and image contents are absent from ordinary logs.</x:v>
+        <x:v>Provider focused verification</x:v>
       </x:c>
       <x:c r="D40" s="3" t="str">
-        <x:v>Local development</x:v>
+        <x:v>Isolated Windows development checkout</x:v>
       </x:c>
       <x:c r="E40" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F40" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F40" s="7" t="str">
+        <x:v>work/evidence/cc-t009-provider-focused-3.xml</x:v>
+      </x:c>
       <x:c r="G40" s="7" t="str">
-        <x:v>Planned evidence requirement; no result has been observed by this tracker builder.</x:v>
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
       </x:c>
       <x:c r="H40" s="3" t="str">
         <x:v>Execution</x:v>
@@ -17057,19 +17343,36 @@
       <x:c r="J40" s="3" t="str">
         <x:v>["CC-T009-S03"]</x:v>
       </x:c>
-      <x:c r="K40" s="7" t="str"/>
-      <x:c r="L40" s="8" t="str"/>
-      <x:c r="M40" s="7" t="str"/>
-      <x:c r="N40" s="7" t="str"/>
-      <x:c r="O40" s="7" t="str"/>
+      <x:c r="K40" s="7" t="str">
+        <x:v>93cd1df77083e1c81a4e5ac0df4e6def5a7dcf336afc772e6c8309107ae5f0c2</x:v>
+      </x:c>
+      <x:c r="L40" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="M40" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
+      </x:c>
+      <x:c r="N40" s="7" t="str">
+        <x:v>.venv/Scripts/python.exe -m pytest -q tests/test_provider_conformance.py --junitxml=../evidence/cc-t009-provider-focused-3.xml</x:v>
+      </x:c>
+      <x:c r="O40" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="P40" s="3" t="str">
-        <x:v>python -m pytest -q tests/acceptance/test_provider_conformance.py
-All applicable acceptance criteria pass; separately record manual-source, hardware or clean-installation observations when required.</x:v>
-      </x:c>
-      <x:c r="Q40" s="7" t="str"/>
-      <x:c r="R40" s="7" t="str"/>
-      <x:c r="S40" s="7" t="str"/>
-      <x:c r="T40" s="7" t="str"/>
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
+      </x:c>
+      <x:c r="Q40" s="7" t="str">
+        <x:v>32 passed, 72 subtests passed.</x:v>
+      </x:c>
+      <x:c r="R40" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
+      <x:c r="S40" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="T40" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
       <x:c r="U40" s="7" t="str"/>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
@@ -22479,23 +22782,393 @@
       </x:c>
       <x:c r="U154" s="7" t="str"/>
     </x:row>
+    <x:row r="155" ht="54" customHeight="1">
+      <x:c r="A155" s="3" t="str">
+        <x:v>CC-E154</x:v>
+      </x:c>
+      <x:c r="B155" s="3" t="str">
+        <x:v>Resume authorization and checkpoint reconciliation</x:v>
+      </x:c>
+      <x:c r="C155" s="3" t="str">
+        <x:v>Saved project workbook and preserved planning input hashes reconciled.</x:v>
+      </x:c>
+      <x:c r="D155" s="3" t="str">
+        <x:v>Local development</x:v>
+      </x:c>
+      <x:c r="E155" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F155" s="7" t="str">
+        <x:v>work/evidence/resume-20260912.md</x:v>
+      </x:c>
+      <x:c r="G155" s="7" t="str">
+        <x:v>Planning observation only; not an engineering acceptance result.</x:v>
+      </x:c>
+      <x:c r="H155" s="3" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+      <x:c r="I155" s="3" t="str">
+        <x:v>["CC-T003","CC-T009"]</x:v>
+      </x:c>
+      <x:c r="J155" s="3" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="K155" s="7" t="str">
+        <x:v>87aa45fc1e96070c8dab2a8ff00fc9b03d637b95be157fd5697376dfba28c379</x:v>
+      </x:c>
+      <x:c r="L155" s="8" t="n">
+        <x:v>46277.745404166664</x:v>
+      </x:c>
+      <x:c r="M155" s="7" t="str"/>
+      <x:c r="N155" s="7" t="str"/>
+      <x:c r="O155" s="7" t="str"/>
+      <x:c r="P155" s="3" t="str">
+        <x:v>Resume exact saved project state without overwriting external changes.</x:v>
+      </x:c>
+      <x:c r="Q155" s="7" t="str">
+        <x:v>User hold superseded. Existing project tracker and branch restored as execution baseline. Changed Downloads template left untouched.</x:v>
+      </x:c>
+      <x:c r="R155" s="7" t="str">
+        <x:v>7dcc5f05015e8a995e37eb9eea46f683318bf7d9</x:v>
+      </x:c>
+      <x:c r="S155" s="7" t="str">
+        <x:v>CC-RUN-resume-20260912</x:v>
+      </x:c>
+      <x:c r="T155" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
+      <x:c r="U155" s="7" t="str"/>
+    </x:row>
+    <x:row r="156" ht="54" customHeight="1">
+      <x:c r="A156" s="3" t="str">
+        <x:v>CC-E155</x:v>
+      </x:c>
+      <x:c r="B156" s="3" t="str">
+        <x:v>Remote source and stale Excel reconciliation</x:v>
+      </x:c>
+      <x:c r="C156" s="3" t="str">
+        <x:v>Remote source and stale Excel reconciliation</x:v>
+      </x:c>
+      <x:c r="D156" s="3" t="str">
+        <x:v>Isolated Windows development checkout</x:v>
+      </x:c>
+      <x:c r="E156" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F156" s="7" t="str">
+        <x:v>work/evidence/remote-checkpoint-reconciliation-20260912.md</x:v>
+      </x:c>
+      <x:c r="G156" s="7" t="str">
+        <x:v>Partial task evidence. Does not mark all affected tasks complete.</x:v>
+      </x:c>
+      <x:c r="H156" s="3" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="I156" s="3" t="str">
+        <x:v>["CC-T003","CC-T009","CC-T010","CC-T011","CC-T012"]</x:v>
+      </x:c>
+      <x:c r="J156" s="3" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="K156" s="7" t="str">
+        <x:v>5667b6933d025879256fe42b7be581d8afec32458a3bcf656cfe7c4665a7f6c5</x:v>
+      </x:c>
+      <x:c r="L156" s="8" t="n">
+        <x:v>46277.75174638889</x:v>
+      </x:c>
+      <x:c r="M156" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1</x:v>
+      </x:c>
+      <x:c r="N156" s="7" t="str">
+        <x:v>git fetch; git diff; saved workbook/hash inspection</x:v>
+      </x:c>
+      <x:c r="O156" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P156" s="3" t="str">
+        <x:v>Preserve remote work and verify existing acceptance fixtures.</x:v>
+      </x:c>
+      <x:c r="Q156" s="7" t="str">
+        <x:v>114 passed, 1 skipped, 92 subtests passed. Full task gates still require review and missing integration evidence.</x:v>
+      </x:c>
+      <x:c r="R156" s="7" t="str">
+        <x:v>d9d94ed854198b9c0252dcfdaf3b5afccb06c217</x:v>
+      </x:c>
+      <x:c r="S156" s="7" t="str">
+        <x:v>CC-RUN-remote-reconcile-20260912</x:v>
+      </x:c>
+      <x:c r="T156" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
+      <x:c r="U156" s="7" t="str"/>
+    </x:row>
+    <x:row r="157" ht="54" customHeight="1">
+      <x:c r="A157" s="3" t="str">
+        <x:v>CC-E156</x:v>
+      </x:c>
+      <x:c r="B157" s="3" t="str">
+        <x:v>Fresh full-suite verification of remote checkpoint</x:v>
+      </x:c>
+      <x:c r="C157" s="3" t="str">
+        <x:v>Fresh full-suite verification of remote checkpoint</x:v>
+      </x:c>
+      <x:c r="D157" s="3" t="str">
+        <x:v>Isolated Windows development checkout</x:v>
+      </x:c>
+      <x:c r="E157" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F157" s="7" t="str">
+        <x:v>work/evidence/reconciled-remote-baseline-20260912.xml</x:v>
+      </x:c>
+      <x:c r="G157" s="7" t="str">
+        <x:v>Partial task evidence. Does not mark all affected tasks complete.</x:v>
+      </x:c>
+      <x:c r="H157" s="3" t="str">
+        <x:v>Execution</x:v>
+      </x:c>
+      <x:c r="I157" s="3" t="str">
+        <x:v>["CC-T003","CC-T009","CC-T010","CC-T011","CC-T012"]</x:v>
+      </x:c>
+      <x:c r="J157" s="3" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="K157" s="7" t="str">
+        <x:v>702ea3844a7a7152637345cfdf6e9781baf4aa869df2ae14cb8d689a67cd7652</x:v>
+      </x:c>
+      <x:c r="L157" s="8" t="n">
+        <x:v>46277.75174638889</x:v>
+      </x:c>
+      <x:c r="M157" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1</x:v>
+      </x:c>
+      <x:c r="N157" s="7" t="str">
+        <x:v>python -m pytest -q tests --junitxml=../evidence/reconciled-remote-baseline-20260912.xml</x:v>
+      </x:c>
+      <x:c r="O157" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P157" s="3" t="str">
+        <x:v>Preserve remote work and verify existing acceptance fixtures.</x:v>
+      </x:c>
+      <x:c r="Q157" s="7" t="str">
+        <x:v>114 passed, 1 skipped, 92 subtests passed. Full task gates still require review and missing integration evidence.</x:v>
+      </x:c>
+      <x:c r="R157" s="7" t="str">
+        <x:v>d9d94ed854198b9c0252dcfdaf3b5afccb06c217</x:v>
+      </x:c>
+      <x:c r="S157" s="7" t="str">
+        <x:v>CC-RUN-remote-reconcile-20260912</x:v>
+      </x:c>
+      <x:c r="T157" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
+      <x:c r="U157" s="7" t="str"/>
+    </x:row>
+    <x:row r="158" ht="54" customHeight="1">
+      <x:c r="A158" s="3" t="str">
+        <x:v>CC-E157</x:v>
+      </x:c>
+      <x:c r="B158" s="3" t="str">
+        <x:v>Full resumed application suite</x:v>
+      </x:c>
+      <x:c r="C158" s="3" t="str">
+        <x:v>Full resumed application suite</x:v>
+      </x:c>
+      <x:c r="D158" s="3" t="str">
+        <x:v>Isolated Windows development checkout</x:v>
+      </x:c>
+      <x:c r="E158" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F158" s="7" t="str">
+        <x:v>work/evidence/resume-direct-full-suite-20260912.xml</x:v>
+      </x:c>
+      <x:c r="G158" s="7" t="str">
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
+      </x:c>
+      <x:c r="H158" s="3" t="str">
+        <x:v>Execution</x:v>
+      </x:c>
+      <x:c r="I158" s="3" t="str">
+        <x:v>["CC-T003", "CC-T009", "CC-T010", "CC-T011", "CC-T012"]</x:v>
+      </x:c>
+      <x:c r="J158" s="3" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="K158" s="7" t="str">
+        <x:v>07771e534e7bbcc368cc9157d3f322073f9cad4710aa46e66c0e2226f458e434</x:v>
+      </x:c>
+      <x:c r="L158" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="M158" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
+      </x:c>
+      <x:c r="N158" s="7" t="str">
+        <x:v>.venv/Scripts/python.exe -m pytest -q --junitxml=../evidence/resume-direct-full-suite-20260912.xml</x:v>
+      </x:c>
+      <x:c r="O158" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P158" s="3" t="str">
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
+      </x:c>
+      <x:c r="Q158" s="7" t="str">
+        <x:v>141 passed, 1 skipped, 108 subtests passed.</x:v>
+      </x:c>
+      <x:c r="R158" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
+      <x:c r="S158" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="T158" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
+      <x:c r="U158" s="7" t="str"/>
+    </x:row>
+    <x:row r="159" ht="60" customHeight="1">
+      <x:c r="A159" s="3" t="str">
+        <x:v>CC-E158</x:v>
+      </x:c>
+      <x:c r="B159" s="3" t="str">
+        <x:v>Focused model asset, sidecar and inference settings fixtures</x:v>
+      </x:c>
+      <x:c r="C159" s="3" t="str">
+        <x:v>Focused model asset, sidecar and inference settings fixtures</x:v>
+      </x:c>
+      <x:c r="D159" s="3" t="str">
+        <x:v>Isolated Windows development checkout</x:v>
+      </x:c>
+      <x:c r="E159" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F159" s="7" t="str">
+        <x:v>work/evidence/cc-t010-t011-t012-runtime-focused.xml</x:v>
+      </x:c>
+      <x:c r="G159" s="7" t="str">
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
+      </x:c>
+      <x:c r="H159" s="3" t="str">
+        <x:v>Execution</x:v>
+      </x:c>
+      <x:c r="I159" s="3" t="str">
+        <x:v>["CC-T010", "CC-T011", "CC-T012"]</x:v>
+      </x:c>
+      <x:c r="J159" s="3" t="str">
+        <x:v>["CC-T010-S03", "CC-T011-S03", "CC-T012-S03"]</x:v>
+      </x:c>
+      <x:c r="K159" s="7" t="str">
+        <x:v>746d7dbc2f1ede92a054c3a7b3f89c9831f5fb39cae6d45d3e16e6fc0b53055b</x:v>
+      </x:c>
+      <x:c r="L159" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="M159" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
+      </x:c>
+      <x:c r="N159" s="7" t="str">
+        <x:v>.venv/Scripts/python.exe -m pytest -q tests/acceptance/test_model_assets.py tests/acceptance/test_sidecar_lifecycle.py tests/acceptance/test_inference_settings.py --junitxml=../evidence/cc-t010-t011-t012-runtime-focused.xml</x:v>
+      </x:c>
+      <x:c r="O159" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P159" s="3" t="str">
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
+      </x:c>
+      <x:c r="Q159" s="7" t="str">
+        <x:v>29 passed, 12 subtests passed. Evidence remains synthetic and does not prove real model/runtime/hardware activation.</x:v>
+      </x:c>
+      <x:c r="R159" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
+      <x:c r="S159" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="T159" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
+      <x:c r="U159" s="7" t="str"/>
+    </x:row>
+    <x:row r="160" ht="54" customHeight="1">
+      <x:c r="A160" s="3" t="str">
+        <x:v>CC-E159</x:v>
+      </x:c>
+      <x:c r="B160" s="3" t="str">
+        <x:v>Coordinator implementation checkpoint and known limits</x:v>
+      </x:c>
+      <x:c r="C160" s="3" t="str">
+        <x:v>Coordinator implementation checkpoint and known limits</x:v>
+      </x:c>
+      <x:c r="D160" s="3" t="str">
+        <x:v>Isolated Windows development checkout</x:v>
+      </x:c>
+      <x:c r="E160" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F160" s="7" t="str">
+        <x:v>work/evidence/resume-direct-implementation-20260912.md</x:v>
+      </x:c>
+      <x:c r="G160" s="7" t="str">
+        <x:v>Resumed implementation evidence. Task closure still depends on review and any non-synthetic gates named in the plan.</x:v>
+      </x:c>
+      <x:c r="H160" s="3" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="I160" s="3" t="str">
+        <x:v>["CC-T003", "CC-T009", "CC-T010", "CC-T011", "CC-T012"]</x:v>
+      </x:c>
+      <x:c r="J160" s="3" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="K160" s="7" t="str">
+        <x:v>574a228abb994a8033b853eb69e99822ae6ca3949ed013f2c3ba95e11dd30fbd</x:v>
+      </x:c>
+      <x:c r="L160" s="8" t="n">
+        <x:v>46277.97015940972</x:v>
+      </x:c>
+      <x:c r="M160" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows</x:v>
+      </x:c>
+      <x:c r="N160" s="7" t="str"/>
+      <x:c r="O160" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P160" s="3" t="str">
+        <x:v>Focused and full verification evidence is recorded without claiming unperformed hardware, model-load or pilot-source gates.</x:v>
+      </x:c>
+      <x:c r="Q160" s="7" t="str">
+        <x:v>Verified source commit 933a392. T003/T009 review steps remain open; T010-T012 real asset/runtime gates remain unperformed.</x:v>
+      </x:c>
+      <x:c r="R160" s="7" t="str">
+        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+      </x:c>
+      <x:c r="S160" s="7" t="str">
+        <x:v>CC-RUN-resume-direct-20260912</x:v>
+      </x:c>
+      <x:c r="T160" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
+      <x:c r="U160" s="7" t="str"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E2:E154">
+  <x:conditionalFormatting sqref="E2:E160">
     <x:cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Blocked"/>
     <x:cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="In progress"/>
     <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="E2:E154">
+    <x:dataValidation type="list" sqref="E2:E160">
       <x:formula1>"Not started,In progress,Blocked,Done,Skipped,N/A"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="H2:H154">
+    <x:dataValidation type="list" sqref="H2:H160">
       <x:formula1>"Source,Research,Design,Execution,Review,Release,Decision"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2b0303daae54b8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1f361bcb1134f01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update Automotive RAG tracker after review fixes
</commit_message>
<xml_diff>
--- a/docs/automotive-rag/CC_Workshop_Planning_Tracker.xlsx
+++ b/docs/automotive-rag/CC_Workshop_Planning_Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6c9c1fd084704e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handover" sheetId="2" r:id="Re28694cb5a9e40dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" r:id="R263f41c557d34543"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="4" r:id="Rcc5521ff0beb454b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="5" r:id="Rfe27f61c23b145a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="6" r:id="Rdf921ca139d64f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R178323e63cc441c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handover" sheetId="2" r:id="Rb1c5b839c20f44e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" r:id="Rb5d081017aa945e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="4" r:id="R7ec6562d12d94bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="5" r:id="R2e6e147b23064637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="6" r:id="R689799c6eb34433e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -315,7 +315,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblEvidence" displayName="tblEvidence" ref="A1:U160" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblEvidence" displayName="tblEvidence" ref="A1:U163" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="#"/>
     <x:tableColumn id="2" name="Evidence required"/>
@@ -577,7 +577,7 @@
         <x:v>Snapshot ID</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>CC-SNAPSHOT-20260912231714290-fc76223c</x:v>
+        <x:v>CC-SNAPSHOT-20260914120341144-0acc14d6</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26" customHeight="1">
@@ -585,7 +585,7 @@
         <x:v>Updated UTC</x:v>
       </x:c>
       <x:c r="B6" s="15" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
@@ -707,7 +707,7 @@
         <x:v>Implementation state</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
-        <x:v>CC-T000: Done. Initial engineering tasks Done: 1 of 31. Only recorded acceptance evidence justifies completion.</x:v>
+        <x:v>CC-T000: Done. Initial engineering tasks Done: 3 of 31. Only recorded acceptance evidence justifies completion.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
@@ -731,7 +731,7 @@
       </x:c>
       <x:c r="B24" s="11" t="n">
         <x:f>COUNTIFS(tblTasks[Work class],"Engineering",tblTasks[Release],"Initial",tblTasks[Status],"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
@@ -740,7 +740,7 @@
       </x:c>
       <x:c r="B25" s="11" t="n">
         <x:f>COUNTIFS(tblTasks[Work class],"Engineering",tblTasks[Release],"Initial",tblTasks[Status],"In progress")</x:f>
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
@@ -767,7 +767,7 @@
       </x:c>
       <x:c r="B28" s="12" t="n">
         <x:f>IF(B23=0,0,B24/B23)</x:f>
-        <x:v>0.03225806451612903</x:v>
+        <x:v>0.0967741935483871</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
@@ -785,7 +785,7 @@
       </x:c>
       <x:c r="B30" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Work class],"Engineering",tblSteps[Release],"Initial",tblSteps[Status],"Done")</x:f>
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
@@ -803,7 +803,7 @@
       </x:c>
       <x:c r="B32" s="12" t="n">
         <x:f>IF(B29=0,0,B30/B29)</x:f>
-        <x:v>0.08064516129032258</x:v>
+        <x:v>0.0967741935483871</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
@@ -839,7 +839,7 @@
       </x:c>
       <x:c r="B36" s="11" t="n">
         <x:f>COUNTIF(tblDecisions[Status],"Open")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
@@ -884,7 +884,7 @@
       </x:c>
       <x:c r="B41" s="11" t="n">
         <x:f>COUNTIFS(tblEvidence[Evidence kind],"Execution",tblEvidence[Status],"Done")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
@@ -893,7 +893,7 @@
       </x:c>
       <x:c r="B42" s="11" t="n">
         <x:f>COUNTIFS(tblEvidence[Evidence kind],"Review",tblEvidence[Status],"Done")</x:f>
-        <x:v>6</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
@@ -911,7 +911,7 @@
       </x:c>
       <x:c r="B44" s="11" t="n">
         <x:f>COUNTIFS(tblEvidence[Evidence kind],"Decision",tblEvidence[Status],"Done")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -972,7 +972,7 @@
         <x:v>Snapshot ID</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>CC-SNAPSHOT-20260912231714290-fc76223c</x:v>
+        <x:v>CC-SNAPSHOT-20260914120341144-0acc14d6</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
@@ -980,7 +980,7 @@
         <x:v>Previous snapshot ID</x:v>
       </x:c>
       <x:c r="B8" s="7" t="str">
-        <x:v>CC-SNAPSHOT-20260912180231622-e8a8cf42</x:v>
+        <x:v>CC-SNAPSHOT-20260914115438499-8f7e3a4a</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
@@ -988,7 +988,7 @@
         <x:v>Last update UTC</x:v>
       </x:c>
       <x:c r="B9" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26" customHeight="1">
@@ -1020,7 +1020,7 @@
         <x:v>Actual HEAD</x:v>
       </x:c>
       <x:c r="B13" s="7" t="str">
-        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="26" customHeight="1">
@@ -1028,7 +1028,7 @@
         <x:v>Current task</x:v>
       </x:c>
       <x:c r="B14" s="7" t="str">
-        <x:v>CC-T003; CC-T009; CC-T010-CC-T012 follow-up review</x:v>
+        <x:v>CC-T004 or CC-T005</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -1036,15 +1036,15 @@
         <x:v>Current step</x:v>
       </x:c>
       <x:c r="B15" s="7" t="str">
-        <x:v>CC-T003-S04 and CC-T009-S04</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="38" customHeight="1">
+        <x:v>Select next ready task after CC-T003 and CC-T009 closure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="26" customHeight="1">
       <x:c r="A16" s="17" t="str">
         <x:v>Last verified execution</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
-        <x:v>Full resumed suite: 141 passed, 1 skipped, 108 subtests passed. Focused Garage: 30 passed, 1 skipped, 24 subtests. Provider: 32 passed, 72 subtests. Runtime/model/settings fixtures: 29 passed, 12 subtests.</x:v>
+        <x:v>Reviewer-fix focused suite: 81 passed, 1 skipped, 104 subtests. Full suite: 150 passed, 1 skipped, 112 subtests.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="26" customHeight="1">
@@ -1052,7 +1052,7 @@
         <x:v>Last verified evidence IDs</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
-        <x:v>["CC-E013", "CC-E014", "CC-E015", "CC-E037", "CC-E038", "CC-E039", "CC-E157", "CC-E158", "CC-E159"]</x:v>
+        <x:v>["CC-E016", "CC-E040", "CC-E161", "CC-E162"]</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="26" customHeight="1">
@@ -1060,7 +1060,7 @@
         <x:v>Ready next tasks</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>["CC-T003","CC-T009"]</x:v>
+        <x:v>["CC-T004","CC-T005","CC-T010"]</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="38" customHeight="1">
@@ -1092,7 +1092,7 @@
         <x:v>Files changed this session</x:v>
       </x:c>
       <x:c r="B22" s="7" t="str">
-        <x:v>Source commit 933a392 plus regenerated tracker, JSON snapshot and handover artifacts.</x:v>
+        <x:v>Source commit 1e87202 plus regenerated tracker, JSON snapshot, handover and evidence artifacts.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
@@ -1100,7 +1100,7 @@
         <x:v>Uncommitted and unpublished state</x:v>
       </x:c>
       <x:c r="B23" s="7" t="str">
-        <x:v>Tracker/doc artifact update is being prepared after source commit 933a392. No GitHub push has been claimed yet.</x:v>
+        <x:v>Tracker/docs checkpoint still needs to be synced and pushed after workbook regeneration.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
@@ -1108,7 +1108,7 @@
         <x:v>Next concrete action</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
-        <x:v>Complete final review for CC-T003 and CC-T009, then proceed to CC-T004 or CC-T005 once tracker handover is synced.</x:v>
+        <x:v>Proceed to CC-T004 vehicle profiles/applicability or CC-T005 source provenance. For any compiled software edition, bump the version number, commit and push the source, compile the artifact, and record version/build evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
@@ -1116,7 +1116,7 @@
         <x:v>Expected result</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
-        <x:v>Workbook, JSON and GitHub branch identify source commit 933a392 and distinguish synthetic fixture evidence from real runtime/model/hardware gates.</x:v>
+        <x:v>CC-T003 and CC-T009 are closed with reviewer-fix evidence; versioning rule CC-D014 remains active for compiled releases.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="26" customHeight="1">
@@ -1124,7 +1124,7 @@
         <x:v>Stop condition</x:v>
       </x:c>
       <x:c r="B26" s="7" t="str">
-        <x:v>Do not close T010, T011 or T012 until real asset/runtime gates in the plan are satisfied or explicitly deferred.</x:v>
+        <x:v>Do not close CC-T010, CC-T011 or CC-T012 until real model/runtime gates are satisfied or explicitly deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="26" customHeight="1">
@@ -1615,7 +1615,7 @@
         <x:v>Local development</x:v>
       </x:c>
       <x:c r="E6" s="7" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F6" s="7" t="str">
         <x:v>Coordinator</x:v>
@@ -1627,7 +1627,7 @@
         <x:v>garage_isolation: complete acceptance and review evidence</x:v>
       </x:c>
       <x:c r="I6" s="7" t="str">
-        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
       </x:c>
       <x:c r="J6" s="3" t="str">
         <x:v>1. Add Garage registry and creation/read/update operations.
@@ -1637,7 +1637,7 @@
 5. Add scoped file resolution and single-instance storage ownership.</x:v>
       </x:c>
       <x:c r="K6" s="7" t="str">
-        <x:v>Implementation and focused verification now pass from source commit 933a392. Final review/handover step remains open before task closure.</x:v>
+        <x:v>Closed after independent review findings were fixed in commit 1e87202. Fresh focused and full-suite verification passed; Windows directory-link escape fixture remains skipped because this account lacks link creation rights.</x:v>
       </x:c>
       <x:c r="L6" s="3" t="str">
         <x:v>Engineering</x:v>
@@ -1676,7 +1676,7 @@
       </x:c>
       <x:c r="V6" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"Done")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W6" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"Skipped")+COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"N/A")</x:f>
@@ -1684,17 +1684,17 @@
       </x:c>
       <x:c r="X6" s="12" t="n">
         <x:f>IF([@Step total]=0,0,([@Steps done]+[@Steps waived])/[@Step total])</x:f>
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y6" s="12" t="n">
         <x:f>IF([@Step total]=0,0,[@Steps done]/[@Step total])</x:f>
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Z6" s="7" t="str">
-        <x:v>Not evaluated</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="AA6" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="AB6" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -2172,7 +2172,7 @@
         <x:v>Local development</x:v>
       </x:c>
       <x:c r="E12" s="7" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F12" s="7" t="str">
         <x:v>Coordinator</x:v>
@@ -2184,7 +2184,7 @@
         <x:v>provider_conformance: complete acceptance and review evidence</x:v>
       </x:c>
       <x:c r="I12" s="7" t="str">
-        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
         <x:v>1. Implement the OpenAI-compatible transport subset.
@@ -2194,7 +2194,7 @@
 5. Prevent cloud endpoints under the chosen network policy.</x:v>
       </x:c>
       <x:c r="K12" s="7" t="str">
-        <x:v>Implementation and focused verification now pass from source commit 933a392. Final review/handover step remains open before task closure.</x:v>
+        <x:v>Closed after independent review findings were fixed in commit 1e87202. Fresh focused and full-suite verification passed; real llama.cpp/model certification remains in later tasks.</x:v>
       </x:c>
       <x:c r="L12" s="3" t="str">
         <x:v>Engineering</x:v>
@@ -2233,7 +2233,7 @@
       </x:c>
       <x:c r="V12" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"Done")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="W12" s="11" t="n">
         <x:f>COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"Skipped")+COUNTIFS(tblSteps[Task],[@Task],tblSteps[Status],"N/A")</x:f>
@@ -2241,17 +2241,17 @@
       </x:c>
       <x:c r="X12" s="12" t="n">
         <x:f>IF([@Step total]=0,0,([@Steps done]+[@Steps waived])/[@Step total])</x:f>
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Y12" s="12" t="n">
         <x:f>IF([@Step total]=0,0,[@Steps done]/[@Step total])</x:f>
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Z12" s="7" t="str">
-        <x:v>Not evaluated</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="AA12" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="AB12" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -2349,7 +2349,7 @@
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="AA13" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="AB13" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -2449,7 +2449,7 @@
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="AA14" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="AB14" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -2548,7 +2548,7 @@
         <x:v>Not evaluated</x:v>
       </x:c>
       <x:c r="AA15" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="AB15" s="3" t="str">
         <x:f>IF(AND([@Status]="Done",OR([@Step total]=0,[@Closed step ratio]&lt;&gt;1,[@Gate state]&lt;&gt;"Passed")),"Review completion","")</x:f>
@@ -4693,7 +4693,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd4463e6aa5c412f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fa16eec640643b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5750,7 +5750,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t003--implement-the-garage-storage-boundary</x:v>
       </x:c>
       <x:c r="R14" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S14" s="8" t="n">
         <x:v>46277.745404166664</x:v>
@@ -5833,7 +5833,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t003--implement-the-garage-storage-boundary</x:v>
       </x:c>
       <x:c r="R15" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S15" s="8" t="str"/>
       <x:c r="T15" s="8" t="n">
@@ -5915,7 +5915,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t003--implement-the-garage-storage-boundary</x:v>
       </x:c>
       <x:c r="R16" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S16" s="8" t="str"/>
       <x:c r="T16" s="8" t="n">
@@ -5948,7 +5948,7 @@
         <x:v>Review implement the garage storage boundary, reconcile its evidence and handover, and record the commit if one is created.</x:v>
       </x:c>
       <x:c r="E17" s="7" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F17" s="7" t="str">
         <x:v>Coordinator</x:v>
@@ -5985,23 +5985,25 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t003--implement-the-garage-storage-boundary</x:v>
       </x:c>
       <x:c r="R17" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S17" s="8" t="n">
         <x:v>46277.97015940972</x:v>
       </x:c>
-      <x:c r="T17" s="8" t="str"/>
+      <x:c r="T17" s="8" t="n">
+        <x:v>46279.506944444445</x:v>
+      </x:c>
       <x:c r="U17" s="7" t="str">
-        <x:v>CC-RUN-resume-direct-20260912</x:v>
+        <x:v>CC-RUN-reviewer-fixes-20260914</x:v>
       </x:c>
       <x:c r="V17" s="7" t="str">
-        <x:v>Review and tracker reconciliation started; task is not closed until review evidence is attached.</x:v>
+        <x:v>Independent reviewer findings were addressed, focused reviewer-fix verification passed, full suite passed, and tracker evidence was reconciled.</x:v>
       </x:c>
       <x:c r="W17" s="7" t="str">
-        <x:v>CC-RUN-resume-direct-20260912</x:v>
+        <x:v>CC-RUN-reviewer-fixes-20260914</x:v>
       </x:c>
       <x:c r="X17" s="7" t="str">
-        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="96" customHeight="1">
@@ -7354,7 +7356,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t009--implement-the-inference-provider-contract</x:v>
       </x:c>
       <x:c r="R38" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S38" s="8" t="n">
         <x:v>46277.745404166664</x:v>
@@ -7437,7 +7439,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t009--implement-the-inference-provider-contract</x:v>
       </x:c>
       <x:c r="R39" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S39" s="8" t="str"/>
       <x:c r="T39" s="8" t="n">
@@ -7519,7 +7521,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t009--implement-the-inference-provider-contract</x:v>
       </x:c>
       <x:c r="R40" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S40" s="8" t="str"/>
       <x:c r="T40" s="8" t="n">
@@ -7552,7 +7554,7 @@
         <x:v>Review implement the inference provider contract, reconcile its evidence and handover, and record the commit if one is created.</x:v>
       </x:c>
       <x:c r="E41" s="7" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F41" s="7" t="str">
         <x:v>Coordinator</x:v>
@@ -7589,23 +7591,25 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t009--implement-the-inference-provider-contract</x:v>
       </x:c>
       <x:c r="R41" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S41" s="8" t="n">
         <x:v>46277.97015940972</x:v>
       </x:c>
-      <x:c r="T41" s="8" t="str"/>
+      <x:c r="T41" s="8" t="n">
+        <x:v>46279.506944444445</x:v>
+      </x:c>
       <x:c r="U41" s="7" t="str">
-        <x:v>CC-RUN-resume-direct-20260912</x:v>
+        <x:v>CC-RUN-reviewer-fixes-20260914</x:v>
       </x:c>
       <x:c r="V41" s="7" t="str">
-        <x:v>Review and tracker reconciliation started; task is not closed until review evidence is attached.</x:v>
+        <x:v>Independent reviewer findings were addressed, focused reviewer-fix verification passed, full suite passed, and tracker evidence was reconciled.</x:v>
       </x:c>
       <x:c r="W41" s="7" t="str">
-        <x:v>CC-RUN-resume-direct-20260912</x:v>
+        <x:v>CC-RUN-reviewer-fixes-20260914</x:v>
       </x:c>
       <x:c r="X41" s="7" t="str">
-        <x:v>933a39204a90ff60d26c96444de66dc379e31065</x:v>
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="96" customHeight="1">
@@ -7811,7 +7815,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t010--add-model-assets-and-hardware-discovery</x:v>
       </x:c>
       <x:c r="R44" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S44" s="8" t="n">
         <x:v>46277.97015940972</x:v>
@@ -8097,7 +8101,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t011--supervise-bundled-llamacpp</x:v>
       </x:c>
       <x:c r="R48" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S48" s="8" t="n">
         <x:v>46277.97015940972</x:v>
@@ -8381,7 +8385,7 @@
         <x:v>CC_Workshop_Implementation_Plan.md#cc-t012--add-hardware-controls-and-alternative-local-endpoints</x:v>
       </x:c>
       <x:c r="R52" s="8" t="n">
-        <x:v>46277.970304282404</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="S52" s="8" t="n">
         <x:v>46277.97015940972</x:v>
@@ -14423,7 +14427,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c0c32146eee4590"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69771119efe349ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15023,45 +15027,49 @@
         <x:v>Source</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="54" customHeight="1">
+    <x:row r="15" ht="84" customHeight="1">
       <x:c r="A15" s="3" t="str">
         <x:v>CC-D014</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
-        <x:v>Confirm actual vehicle VIN, engine code, transmission code and brake PR code for the source-reviewed pilot.</x:v>
+        <x:v>Versioning rule for every compiled software edition</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
-        <x:v>CC-T025 real applicable repair workflow</x:v>
+        <x:v>Release packaging, installer evidence, handover closure and any claim that a compiled software edition has been created.</x:v>
       </x:c>
       <x:c r="D15" s="3" t="str">
-        <x:v>Supply only independently confirmed configuration fields and their evidence.</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="str"/>
+        <x:v>Every software version that is created for this project must advance the application version number before release packaging. A compiled build must record the version, commit SHA, pushed branch, build artifact or installer manifest, and verification evidence in the tracker. A commit or push alone is not a compiled software version; a compiled artifact without a version bump cannot be marked as release evidence.</x:v>
+      </x:c>
+      <x:c r="E15" s="7" t="str">
+        <x:v>Every software version that is created for this project must advance the application version number before release packaging. A compiled build must record the version, commit SHA, pushed branch, build artifact or installer manifest, and verification evidence in the tracker. A commit or push alone is not a compiled software version; a compiled artifact without a version bump cannot be marked as release evidence.</x:v>
+      </x:c>
       <x:c r="F15" s="7" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="G15" s="9" t="str"/>
+        <x:v>Answered</x:v>
+      </x:c>
+      <x:c r="G15" s="9" t="n">
+        <x:v>46279</x:v>
+      </x:c>
       <x:c r="H15" s="3" t="str">
-        <x:v>Vehicle identification</x:v>
+        <x:v>User rule</x:v>
       </x:c>
       <x:c r="I15" s="7" t="str">
-        <x:v>User</x:v>
+        <x:v>Coordinator</x:v>
       </x:c>
       <x:c r="J15" s="3" t="str">
-        <x:v>["CC-T025","CC-T026"]</x:v>
+        <x:v>["CC-T029", "CC-T032"]</x:v>
       </x:c>
       <x:c r="K15" s="3" t="str">
-        <x:v>[]</x:v>
+        <x:v>["CC-E160"]</x:v>
       </x:c>
       <x:c r="L15" s="3" t="str">
-        <x:v>Before approving the real repair pilot</x:v>
+        <x:v>Immediately for every future commit, push and compiled build made for this project.</x:v>
       </x:c>
       <x:c r="M15" s="3" t="str"/>
       <x:c r="N15" s="8" t="n">
-        <x:v>46275.5170659375</x:v>
+        <x:v>46279.50255953704</x:v>
       </x:c>
       <x:c r="O15" s="3" t="str">
-        <x:v>Approved plan input gate</x:v>
+        <x:v>User session</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" customHeight="1">
@@ -15168,7 +15176,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb85c29c981904f8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3273690ccf8242bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16222,25 +16230,27 @@
       </x:c>
       <x:c r="U16" s="7" t="str"/>
     </x:row>
-    <x:row r="17" ht="54" customHeight="1">
+    <x:row r="17" ht="84" customHeight="1">
       <x:c r="A17" s="3" t="str">
         <x:v>CC-E016</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
-        <x:v>CC-T003-S04: Review and handover</x:v>
+        <x:v>CC-T003-S04: Garage boundary review, reviewer fixes and handover</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
-        <x:v>Review findings resolved or explicitly recorded; evidence links valid; tracker consistent; commit field is blank or identifies an actual commit.</x:v>
+        <x:v>Independent review identified active-Garage mismatch and JSON payload issues. Fixes were committed and verified.</x:v>
       </x:c>
       <x:c r="D17" s="3" t="str">
-        <x:v>Local development</x:v>
+        <x:v>Isolated Windows development checkout</x:v>
       </x:c>
       <x:c r="E17" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F17" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F17" s="7" t="str">
+        <x:v>work/evidence/reviewer-fixes-20260914.md</x:v>
+      </x:c>
       <x:c r="G17" s="7" t="str">
-        <x:v>Planned evidence requirement; no result has been observed by this tracker builder.</x:v>
+        <x:v>Source provenance and scoped index work remain separate later tasks.</x:v>
       </x:c>
       <x:c r="H17" s="3" t="str">
         <x:v>Review</x:v>
@@ -16251,18 +16261,36 @@
       <x:c r="J17" s="3" t="str">
         <x:v>["CC-T003-S04"]</x:v>
       </x:c>
-      <x:c r="K17" s="7" t="str"/>
-      <x:c r="L17" s="8" t="str"/>
-      <x:c r="M17" s="7" t="str"/>
-      <x:c r="N17" s="7" t="str"/>
-      <x:c r="O17" s="7" t="str"/>
+      <x:c r="K17" s="7" t="str">
+        <x:v>0ad9259030c68ff02a2e649a14548a927c8a77ac2668b6c95d2973b5eece1a30</x:v>
+      </x:c>
+      <x:c r="L17" s="8" t="n">
+        <x:v>46279.506944444445</x:v>
+      </x:c>
+      <x:c r="M17" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows; Codex desktop</x:v>
+      </x:c>
+      <x:c r="N17" s="7" t="str">
+        <x:v>.venv/Scripts/python.exe -m pytest -q tests/acceptance/test_garage_isolation.py tests/acceptance/test_garage_request_scope.py tests/acceptance/test_runtime_contracts.py tests/test_provider_conformance.py tests/acceptance/test_inference_settings.py --junitxml=../evidence/reviewer-fixes-focused-20260914.xml; .venv/Scripts/python.exe -m pytest -q --junitxml=../evidence/reviewer-fixes-full-suite-20260914.xml</x:v>
+      </x:c>
+      <x:c r="O17" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="P17" s="3" t="str">
-        <x:v>Independent review and all required evidence resolve task acceptance; tracker and handover agree. Record only an existing commit.</x:v>
-      </x:c>
-      <x:c r="Q17" s="7" t="str"/>
-      <x:c r="R17" s="7" t="str"/>
-      <x:c r="S17" s="7" t="str"/>
-      <x:c r="T17" s="7" t="str"/>
+        <x:v>Garage boundary reviewer findings fixed and verified without closing later source-provenance work.</x:v>
+      </x:c>
+      <x:c r="Q17" s="7" t="str">
+        <x:v>Focused reviewer-fix suite passed with 81 passed, 1 skipped, 104 subtests; full suite passed with 150 passed, 1 skipped, 112 subtests.</x:v>
+      </x:c>
+      <x:c r="R17" s="7" t="str">
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
+      </x:c>
+      <x:c r="S17" s="7" t="str">
+        <x:v>CC-RUN-reviewer-fixes-20260914</x:v>
+      </x:c>
+      <x:c r="T17" s="7" t="str">
+        <x:v>Independent reviewer and Coordinator</x:v>
+      </x:c>
       <x:c r="U17" s="7" t="str"/>
     </x:row>
     <x:row r="18" ht="96" customHeight="1">
@@ -17375,25 +17403,27 @@
       </x:c>
       <x:c r="U40" s="7" t="str"/>
     </x:row>
-    <x:row r="41" ht="54" customHeight="1">
+    <x:row r="41" ht="84" customHeight="1">
       <x:c r="A41" s="3" t="str">
         <x:v>CC-E040</x:v>
       </x:c>
       <x:c r="B41" s="3" t="str">
-        <x:v>CC-T009-S04: Review and handover</x:v>
+        <x:v>CC-T009-S04: Provider contract review, reviewer fixes and handover</x:v>
       </x:c>
       <x:c r="C41" s="3" t="str">
-        <x:v>Review findings resolved or explicitly recorded; evidence links valid; tracker consistent; commit field is blank or identifies an actual commit.</x:v>
+        <x:v>Independent review identified provider cancellation, schema probe, stream bound, UTF-8 and legacy-profile issues. Fixes were committed and verified.</x:v>
       </x:c>
       <x:c r="D41" s="3" t="str">
-        <x:v>Local development</x:v>
+        <x:v>Isolated Windows development checkout</x:v>
       </x:c>
       <x:c r="E41" s="7" t="str">
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="F41" s="7" t="str"/>
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F41" s="7" t="str">
+        <x:v>work/evidence/reviewer-fixes-20260914.md</x:v>
+      </x:c>
       <x:c r="G41" s="7" t="str">
-        <x:v>Planned evidence requirement; no result has been observed by this tracker builder.</x:v>
+        <x:v>Real llama.cpp/model runtime certification remains separate in CC-T010 and CC-T011.</x:v>
       </x:c>
       <x:c r="H41" s="3" t="str">
         <x:v>Review</x:v>
@@ -17404,18 +17434,36 @@
       <x:c r="J41" s="3" t="str">
         <x:v>["CC-T009-S04"]</x:v>
       </x:c>
-      <x:c r="K41" s="7" t="str"/>
-      <x:c r="L41" s="8" t="str"/>
-      <x:c r="M41" s="7" t="str"/>
-      <x:c r="N41" s="7" t="str"/>
-      <x:c r="O41" s="7" t="str"/>
+      <x:c r="K41" s="7" t="str">
+        <x:v>0ad9259030c68ff02a2e649a14548a927c8a77ac2668b6c95d2973b5eece1a30</x:v>
+      </x:c>
+      <x:c r="L41" s="8" t="n">
+        <x:v>46279.506944444445</x:v>
+      </x:c>
+      <x:c r="M41" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows; Codex desktop</x:v>
+      </x:c>
+      <x:c r="N41" s="7" t="str">
+        <x:v>.venv/Scripts/python.exe -m pytest -q tests/acceptance/test_garage_isolation.py tests/acceptance/test_garage_request_scope.py tests/acceptance/test_runtime_contracts.py tests/test_provider_conformance.py tests/acceptance/test_inference_settings.py --junitxml=../evidence/reviewer-fixes-focused-20260914.xml; .venv/Scripts/python.exe -m pytest -q --junitxml=../evidence/reviewer-fixes-full-suite-20260914.xml</x:v>
+      </x:c>
+      <x:c r="O41" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="P41" s="3" t="str">
-        <x:v>Independent review and all required evidence resolve task acceptance; tracker and handover agree. Record only an existing commit.</x:v>
-      </x:c>
-      <x:c r="Q41" s="7" t="str"/>
-      <x:c r="R41" s="7" t="str"/>
-      <x:c r="S41" s="7" t="str"/>
-      <x:c r="T41" s="7" t="str"/>
+        <x:v>Provider-contract reviewer findings fixed and verified without claiming real model/runtime gates.</x:v>
+      </x:c>
+      <x:c r="Q41" s="7" t="str">
+        <x:v>Focused reviewer-fix suite passed with 81 passed, 1 skipped, 104 subtests; full suite passed with 150 passed, 1 skipped, 112 subtests.</x:v>
+      </x:c>
+      <x:c r="R41" s="7" t="str">
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
+      </x:c>
+      <x:c r="S41" s="7" t="str">
+        <x:v>CC-RUN-reviewer-fixes-20260914</x:v>
+      </x:c>
+      <x:c r="T41" s="7" t="str">
+        <x:v>Independent reviewer and Coordinator</x:v>
+      </x:c>
       <x:c r="U41" s="7" t="str"/>
     </x:row>
     <x:row r="42" ht="96" customHeight="1">
@@ -23152,23 +23200,208 @@
       </x:c>
       <x:c r="U160" s="7" t="str"/>
     </x:row>
+    <x:row r="161" ht="84" customHeight="1">
+      <x:c r="A161" s="3" t="str">
+        <x:v>CC-E160</x:v>
+      </x:c>
+      <x:c r="B161" s="3" t="str">
+        <x:v>User versioning rule added to tracker</x:v>
+      </x:c>
+      <x:c r="C161" s="3" t="str">
+        <x:v>Every software version that is created for this project must advance the application version number before release packaging. A compiled build must record the version, commit SHA, pushed branch, build artifact or installer manifest, and verification evidence in the tracker. A commit or push alone is not a compiled software version; a compiled artifact without a version bump cannot be marked as release evidence.</x:v>
+      </x:c>
+      <x:c r="D161" s="3" t="str">
+        <x:v>Current Codex task and Automotive RAG tracker</x:v>
+      </x:c>
+      <x:c r="E161" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F161" s="7" t="str">
+        <x:v>outputs/CC_Workshop_Planning_Tracker.xlsx; outputs/CC_Workshop_Implementation_Plan.json</x:v>
+      </x:c>
+      <x:c r="G161" s="7" t="str">
+        <x:v>This evidence records the rule itself. It is not evidence that a compiled software version has already been created.</x:v>
+      </x:c>
+      <x:c r="H161" s="3" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+      <x:c r="I161" s="3" t="str">
+        <x:v>["CC-T029", "CC-T032"]</x:v>
+      </x:c>
+      <x:c r="J161" s="3" t="str">
+        <x:v>[]</x:v>
+      </x:c>
+      <x:c r="K161" s="7" t="str"/>
+      <x:c r="L161" s="8" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="M161" s="7" t="str">
+        <x:v>Codex desktop task; tracker builder</x:v>
+      </x:c>
+      <x:c r="N161" s="7" t="str">
+        <x:v>User requested a versioning rule for every software edition created, committed, pushed and compiled.</x:v>
+      </x:c>
+      <x:c r="O161" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P161" s="3" t="str">
+        <x:v>Tracker contains a durable rule requiring each compiled software edition to advance the version number and record commit, push, build and evidence metadata.</x:v>
+      </x:c>
+      <x:c r="Q161" s="7" t="str">
+        <x:v>Decision CC-D014 and evidence CC-E160 define the version-bump rule and tie it to Windows installation and release handover work.</x:v>
+      </x:c>
+      <x:c r="R161" s="7" t="str"/>
+      <x:c r="S161" s="7" t="str">
+        <x:v>CC-RUN-version-rule-20260914</x:v>
+      </x:c>
+      <x:c r="T161" s="7" t="str">
+        <x:v>User</x:v>
+      </x:c>
+      <x:c r="U161" s="7" t="str"/>
+    </x:row>
+    <x:row r="162" ht="60" customHeight="1">
+      <x:c r="A162" s="3" t="str">
+        <x:v>CC-E161</x:v>
+      </x:c>
+      <x:c r="B162" s="3" t="str">
+        <x:v>Independent reviewer report for CC-T003 and CC-T009</x:v>
+      </x:c>
+      <x:c r="C162" s="3" t="str">
+        <x:v>Read-only review report covering Garage and provider checkpoint findings.</x:v>
+      </x:c>
+      <x:c r="D162" s="3" t="str">
+        <x:v>work/cc-workshop/.superpowers/sdd/CC_Workshop_Implementation_Plan/t003-t009-review-20260914.md</x:v>
+      </x:c>
+      <x:c r="E162" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F162" s="7" t="str">
+        <x:v>work/cc-workshop/.superpowers/sdd/CC_Workshop_Implementation_Plan/t003-t009-review-20260914.md</x:v>
+      </x:c>
+      <x:c r="G162" s="7" t="str">
+        <x:v>This report initially blocked task closure; findings were fixed in source commit 1e87202.</x:v>
+      </x:c>
+      <x:c r="H162" s="3" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="I162" s="3" t="str">
+        <x:v>["CC-T003", "CC-T009"]</x:v>
+      </x:c>
+      <x:c r="J162" s="3" t="str">
+        <x:v>["CC-T003-S04", "CC-T009-S04"]</x:v>
+      </x:c>
+      <x:c r="K162" s="7" t="str">
+        <x:v>046de6b76fbdcb21a8dd98ca131a9509550a4611e069fd836597c4fec63c940e</x:v>
+      </x:c>
+      <x:c r="L162" s="8" t="n">
+        <x:v>46279.506944444445</x:v>
+      </x:c>
+      <x:c r="M162" s="7" t="str">
+        <x:v>Codex reviewer subagent</x:v>
+      </x:c>
+      <x:c r="N162" s="7" t="str">
+        <x:v>Independent code review of d9d94ed..933a392 plus subsequent finding verification.</x:v>
+      </x:c>
+      <x:c r="O162" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P162" s="3" t="str">
+        <x:v>Reviewer identifies any Critical or Important findings before closure.</x:v>
+      </x:c>
+      <x:c r="Q162" s="7" t="str">
+        <x:v>Reviewer identified one Critical and seven Important findings; all applicable findings were addressed before closure.</x:v>
+      </x:c>
+      <x:c r="R162" s="7" t="str">
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
+      </x:c>
+      <x:c r="S162" s="7" t="str">
+        <x:v>CC-RUN-reviewer-fixes-20260914</x:v>
+      </x:c>
+      <x:c r="T162" s="7" t="str">
+        <x:v>review_t003_t009</x:v>
+      </x:c>
+      <x:c r="U162" s="7" t="str"/>
+    </x:row>
+    <x:row r="163" ht="84" customHeight="1">
+      <x:c r="A163" s="3" t="str">
+        <x:v>CC-E162</x:v>
+      </x:c>
+      <x:c r="B163" s="3" t="str">
+        <x:v>Reviewer-fix focused and full-suite execution artifacts</x:v>
+      </x:c>
+      <x:c r="C163" s="3" t="str">
+        <x:v>JUnit reports for focused reviewer-fix verification and the full suite.</x:v>
+      </x:c>
+      <x:c r="D163" s="3" t="str">
+        <x:v>work/evidence/reviewer-fixes-focused-20260914.xml; work/evidence/reviewer-fixes-full-suite-20260914.xml</x:v>
+      </x:c>
+      <x:c r="E163" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F163" s="7" t="str">
+        <x:v>work/evidence/reviewer-fixes-focused-20260914.xml; work/evidence/reviewer-fixes-full-suite-20260914.xml</x:v>
+      </x:c>
+      <x:c r="G163" s="7" t="str">
+        <x:v>The focused report hash is recorded first. The full-suite report hash is recorded in Actual result.</x:v>
+      </x:c>
+      <x:c r="H163" s="3" t="str">
+        <x:v>Execution</x:v>
+      </x:c>
+      <x:c r="I163" s="3" t="str">
+        <x:v>["CC-T003", "CC-T009"]</x:v>
+      </x:c>
+      <x:c r="J163" s="3" t="str">
+        <x:v>["CC-T003-S04", "CC-T009-S04"]</x:v>
+      </x:c>
+      <x:c r="K163" s="7" t="str">
+        <x:v>eef007ebd36d2308752aab1a8e69d5febd5b2b9a8f7390ffa4827c233369a656</x:v>
+      </x:c>
+      <x:c r="L163" s="8" t="n">
+        <x:v>46279.506944444445</x:v>
+      </x:c>
+      <x:c r="M163" s="7" t="str">
+        <x:v>Windows; Python 3.12.14; pytest 9.1.1; Git for Windows; Codex desktop</x:v>
+      </x:c>
+      <x:c r="N163" s="7" t="str">
+        <x:v>.venv/Scripts/python.exe -m pytest -q tests/acceptance/test_garage_isolation.py tests/acceptance/test_garage_request_scope.py tests/acceptance/test_runtime_contracts.py tests/test_provider_conformance.py tests/acceptance/test_inference_settings.py --junitxml=../evidence/reviewer-fixes-focused-20260914.xml; .venv/Scripts/python.exe -m pytest -q --junitxml=../evidence/reviewer-fixes-full-suite-20260914.xml</x:v>
+      </x:c>
+      <x:c r="O163" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P163" s="3" t="str">
+        <x:v>Focused reviewer-fix and full-suite commands pass.</x:v>
+      </x:c>
+      <x:c r="Q163" s="7" t="str">
+        <x:v>Focused: 81 passed, 1 skipped, 104 subtests, sha256=eef007ebd36d2308752aab1a8e69d5febd5b2b9a8f7390ffa4827c233369a656. Full: 150 passed, 1 skipped, 112 subtests, sha256=15694dbda2b1a12bbf862b591b536b4c9c77229c2584c03ab97e0730702faaca.</x:v>
+      </x:c>
+      <x:c r="R163" s="7" t="str">
+        <x:v>1e87202a7ed8923e270090aa87f22a4947a68bcc</x:v>
+      </x:c>
+      <x:c r="S163" s="7" t="str">
+        <x:v>CC-RUN-reviewer-fixes-20260914</x:v>
+      </x:c>
+      <x:c r="T163" s="7" t="str">
+        <x:v>Coordinator</x:v>
+      </x:c>
+      <x:c r="U163" s="7" t="str"/>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E2:E160">
+  <x:conditionalFormatting sqref="E2:E163">
     <x:cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Blocked"/>
     <x:cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="In progress"/>
     <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="E2:E160">
+    <x:dataValidation type="list" sqref="E2:E163">
       <x:formula1>"Not started,In progress,Blocked,Done,Skipped,N/A"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="H2:H160">
+    <x:dataValidation type="list" sqref="H2:H163">
       <x:formula1>"Source,Research,Design,Execution,Review,Release,Decision"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1f361bcb1134f01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51dd0312ae74d97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>